<commit_message>
Record the Commons photo source for every aircraft; document fetch_photos.py
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P5LiqL3Bpjqh9kGwNLAGyt
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chapters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="HandSumRules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Settings" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Archetypes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Routes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="RouteCatalogue" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Aircraft" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Finance" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Airports" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Calendar" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Market" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Events" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Challenges" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Mechanics" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Catering" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Livery" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Hunts" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HandSumRules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archetypes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RouteCatalogue" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aircraft" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Airports" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Challenges" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catering" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livery" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hunts" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29384,7 +29384,11 @@
       <c r="O2" s="23" t="n"/>
       <c r="P2" s="23" t="n"/>
       <c r="Q2" s="23" t="n"/>
-      <c r="R2" s="23" t="n"/>
+      <c r="R2" s="23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:First_Flight_Twin_Otter_Series_400_C-FDHT.jpg</t>
+        </is>
+      </c>
       <c r="S2" s="12" t="inlineStr">
         <is>
           <t>live</t>
@@ -29445,7 +29449,11 @@
       <c r="O3" s="23" t="n"/>
       <c r="P3" s="23" t="n"/>
       <c r="Q3" s="23" t="n"/>
-      <c r="R3" s="23" t="n"/>
+      <c r="R3" s="23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Saab-Fairchild_340_in_flight.jpg</t>
+        </is>
+      </c>
       <c r="S3" s="12" t="inlineStr">
         <is>
           <t>live</t>
@@ -29506,7 +29514,11 @@
       <c r="O4" s="23" t="n"/>
       <c r="P4" s="23" t="n"/>
       <c r="Q4" s="23" t="n"/>
-      <c r="R4" s="23" t="n"/>
+      <c r="R4" s="23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:ATR_72-600_ATR_house_colors_F-WWEY_-_MSN_98_%289742100696%29.jpg</t>
+        </is>
+      </c>
       <c r="S4" s="12" t="inlineStr">
         <is>
           <t>live</t>
@@ -29567,7 +29579,11 @@
       <c r="O5" s="23" t="n"/>
       <c r="P5" s="23" t="n"/>
       <c r="Q5" s="23" t="n"/>
-      <c r="R5" s="23" t="n"/>
+      <c r="R5" s="23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Embraer_190-100_PP-XMB_%286921229367%29.jpg</t>
+        </is>
+      </c>
       <c r="S5" s="12" t="inlineStr">
         <is>
           <t>live</t>
@@ -29628,7 +29644,11 @@
       <c r="O6" s="23" t="n"/>
       <c r="P6" s="23" t="n"/>
       <c r="Q6" s="23" t="n"/>
-      <c r="R6" s="23" t="n"/>
+      <c r="R6" s="23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Bombardier%2C_BD-500_CSeries_CS300%2C_C-FFDK_%2818777967098%29.jpg</t>
+        </is>
+      </c>
       <c r="S6" s="12" t="inlineStr">
         <is>
           <t>live</t>
@@ -29689,7 +29709,11 @@
       <c r="O7" s="23" t="n"/>
       <c r="P7" s="23" t="n"/>
       <c r="Q7" s="23" t="n"/>
-      <c r="R7" s="23" t="n"/>
+      <c r="R7" s="23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:AIB_A320neo_F-WNEW_27may15_LFBO-1.jpg</t>
+        </is>
+      </c>
       <c r="S7" s="12" t="inlineStr">
         <is>
           <t>live</t>
@@ -29750,7 +29774,11 @@
       <c r="O8" s="23" t="n"/>
       <c r="P8" s="23" t="n"/>
       <c r="Q8" s="23" t="n"/>
-      <c r="R8" s="23" t="n"/>
+      <c r="R8" s="23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Boeing%2C_N8701Q%2C_Boeing_737-8_MAX_%282%29.jpg</t>
+        </is>
+      </c>
       <c r="S8" s="12" t="inlineStr">
         <is>
           <t>live</t>
@@ -29807,7 +29835,11 @@
       <c r="O9" s="25" t="n"/>
       <c r="P9" s="25" t="n"/>
       <c r="Q9" s="25" t="n"/>
-      <c r="R9" s="25" t="n"/>
+      <c r="R9" s="25" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:N787BA_01.jpg</t>
+        </is>
+      </c>
       <c r="S9" s="15" t="inlineStr">
         <is>
           <t>later</t>
@@ -29864,7 +29896,11 @@
       <c r="O10" s="25" t="n"/>
       <c r="P10" s="25" t="n"/>
       <c r="Q10" s="25" t="n"/>
-      <c r="R10" s="25" t="n"/>
+      <c r="R10" s="25" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:AIB_A350_F-WXWB_24oct14_LFBO-2.jpg</t>
+        </is>
+      </c>
       <c r="S10" s="15" t="inlineStr">
         <is>
           <t>later</t>
@@ -29921,7 +29957,11 @@
       <c r="O11" s="25" t="n"/>
       <c r="P11" s="25" t="n"/>
       <c r="Q11" s="25" t="n"/>
-      <c r="R11" s="25" t="n"/>
+      <c r="R11" s="25" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Boeing_747-8_first_flight_Everett%2C_WA.jpg</t>
+        </is>
+      </c>
       <c r="S11" s="15" t="inlineStr">
         <is>
           <t>later</t>
@@ -29978,7 +30018,11 @@
       <c r="O12" s="25" t="n"/>
       <c r="P12" s="25" t="n"/>
       <c r="Q12" s="25" t="n"/>
-      <c r="R12" s="25" t="n"/>
+      <c r="R12" s="25" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Airbus_Industrie%2C_F-WWOW%2C_Airbus_A380-841_%2835679929105%29.jpg</t>
+        </is>
+      </c>
       <c r="S12" s="15" t="inlineStr">
         <is>
           <t>later</t>
@@ -30042,6 +30086,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
@@ -30096,7 +30141,11 @@
       <c r="O15" s="23" t="n"/>
       <c r="P15" s="23" t="n"/>
       <c r="Q15" s="23" t="n"/>
-      <c r="R15" s="23" t="n"/>
+      <c r="R15" s="23" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Republic_Airways_N401YX_E75L.jpg</t>
+        </is>
+      </c>
       <c r="S15" s="13" t="inlineStr">
         <is>
           <t>live</t>
@@ -30153,7 +30202,11 @@
       <c r="O16" s="27" t="n"/>
       <c r="P16" s="27" t="n"/>
       <c r="Q16" s="27" t="n"/>
-      <c r="R16" s="27" t="n"/>
+      <c r="R16" s="27" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:N767AN_Boeing_757F_All_White_Colours_%288736741972%29.jpg</t>
+        </is>
+      </c>
       <c r="S16" s="14" t="inlineStr">
         <is>
           <t>placeholder</t>
@@ -30210,7 +30263,11 @@
       <c r="O17" s="25" t="n"/>
       <c r="P17" s="25" t="n"/>
       <c r="Q17" s="25" t="n"/>
-      <c r="R17" s="25" t="n"/>
+      <c r="R17" s="25" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:F-WWCA_A340-642_%28proto%29_Airbus_TLS_09SEP10_%284979496505%29.jpg</t>
+        </is>
+      </c>
       <c r="S17" s="18" t="inlineStr">
         <is>
           <t>later</t>
@@ -30267,13 +30324,18 @@
       <c r="O18" s="25" t="n"/>
       <c r="P18" s="25" t="n"/>
       <c r="Q18" s="25" t="n"/>
-      <c r="R18" s="25" t="n"/>
+      <c r="R18" s="25" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:Boeing_777X_at_Dubai_Airshow_2021_3.jpg</t>
+        </is>
+      </c>
       <c r="S18" s="18" t="inlineStr">
         <is>
           <t>later</t>
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Showroom: real photos of all 15 aircraft from Wikimedia Commons
Fetched with tools/fetch_photos.py: prototypes and demonstrators in maker
colours (an all-white 757; a Republic Airways E175 as Commons has none in
maker colours), each cropped to the card's 3:2 at 900x600 and credited on
the card and in data/Photo-Credits.md. The workbook part now carries
artworkId and the photo columns onto the game's plane list, so each card
shows its photo and each plane paints with its own drawing (every plane
fell back to the Twin Otter drawing before). Docs and screenshot updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P5LiqL3Bpjqh9kGwNLAGyt
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -29381,9 +29381,21 @@
           <t>dhc6</t>
         </is>
       </c>
-      <c r="O2" s="23" t="n"/>
-      <c r="P2" s="23" t="n"/>
-      <c r="Q2" s="23" t="n"/>
+      <c r="O2" s="23" t="inlineStr">
+        <is>
+          <t>dhc6.jpg</t>
+        </is>
+      </c>
+      <c r="P2" s="23" t="inlineStr">
+        <is>
+          <t>Paneuropean</t>
+        </is>
+      </c>
+      <c r="Q2" s="23" t="inlineStr">
+        <is>
+          <t>CC BY-SA 3.0</t>
+        </is>
+      </c>
       <c r="R2" s="23" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:First_Flight_Twin_Otter_Series_400_C-FDHT.jpg</t>
@@ -29446,9 +29458,21 @@
           <t>sf34</t>
         </is>
       </c>
-      <c r="O3" s="23" t="n"/>
-      <c r="P3" s="23" t="n"/>
-      <c r="Q3" s="23" t="n"/>
+      <c r="O3" s="23" t="inlineStr">
+        <is>
+          <t>saab340.jpg</t>
+        </is>
+      </c>
+      <c r="P3" s="23" t="inlineStr">
+        <is>
+          <t>SDASM Archives</t>
+        </is>
+      </c>
+      <c r="Q3" s="23" t="inlineStr">
+        <is>
+          <t>Public domain</t>
+        </is>
+      </c>
       <c r="R3" s="23" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Saab-Fairchild_340_in_flight.jpg</t>
@@ -29511,9 +29535,21 @@
           <t>at72</t>
         </is>
       </c>
-      <c r="O4" s="23" t="n"/>
-      <c r="P4" s="23" t="n"/>
-      <c r="Q4" s="23" t="n"/>
+      <c r="O4" s="23" t="inlineStr">
+        <is>
+          <t>atr72.jpg</t>
+        </is>
+      </c>
+      <c r="P4" s="23" t="inlineStr">
+        <is>
+          <t>Laurent ERRERA</t>
+        </is>
+      </c>
+      <c r="Q4" s="23" t="inlineStr">
+        <is>
+          <t>CC BY-SA 2.0</t>
+        </is>
+      </c>
       <c r="R4" s="23" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:ATR_72-600_ATR_house_colors_F-WWEY_-_MSN_98_%289742100696%29.jpg</t>
@@ -29576,9 +29612,21 @@
           <t>e190</t>
         </is>
       </c>
-      <c r="O5" s="23" t="n"/>
-      <c r="P5" s="23" t="n"/>
-      <c r="Q5" s="23" t="n"/>
+      <c r="O5" s="23" t="inlineStr">
+        <is>
+          <t>e190.jpg</t>
+        </is>
+      </c>
+      <c r="P5" s="23" t="inlineStr">
+        <is>
+          <t>Bob Adams</t>
+        </is>
+      </c>
+      <c r="Q5" s="23" t="inlineStr">
+        <is>
+          <t>CC BY-SA 2.0</t>
+        </is>
+      </c>
       <c r="R5" s="23" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Embraer_190-100_PP-XMB_%286921229367%29.jpg</t>
@@ -29641,9 +29689,21 @@
           <t>narrowbody</t>
         </is>
       </c>
-      <c r="O6" s="23" t="n"/>
-      <c r="P6" s="23" t="n"/>
-      <c r="Q6" s="23" t="n"/>
+      <c r="O6" s="23" t="inlineStr">
+        <is>
+          <t>a220.jpg</t>
+        </is>
+      </c>
+      <c r="P6" s="23" t="inlineStr">
+        <is>
+          <t>Eric Salard</t>
+        </is>
+      </c>
+      <c r="Q6" s="23" t="inlineStr">
+        <is>
+          <t>CC BY-SA 2.0</t>
+        </is>
+      </c>
       <c r="R6" s="23" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Bombardier%2C_BD-500_CSeries_CS300%2C_C-FFDK_%2818777967098%29.jpg</t>
@@ -29706,9 +29766,21 @@
           <t>narrowbody</t>
         </is>
       </c>
-      <c r="O7" s="23" t="n"/>
-      <c r="P7" s="23" t="n"/>
-      <c r="Q7" s="23" t="n"/>
+      <c r="O7" s="23" t="inlineStr">
+        <is>
+          <t>a320.jpg</t>
+        </is>
+      </c>
+      <c r="P7" s="23" t="inlineStr">
+        <is>
+          <t>Gyrostat</t>
+        </is>
+      </c>
+      <c r="Q7" s="23" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0</t>
+        </is>
+      </c>
       <c r="R7" s="23" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:AIB_A320neo_F-WNEW_27may15_LFBO-1.jpg</t>
@@ -29771,9 +29843,21 @@
           <t>narrowbody</t>
         </is>
       </c>
-      <c r="O8" s="23" t="n"/>
-      <c r="P8" s="23" t="n"/>
-      <c r="Q8" s="23" t="n"/>
+      <c r="O8" s="23" t="inlineStr">
+        <is>
+          <t>b737.jpg</t>
+        </is>
+      </c>
+      <c r="P8" s="23" t="inlineStr">
+        <is>
+          <t>John Crowley</t>
+        </is>
+      </c>
+      <c r="Q8" s="23" t="inlineStr">
+        <is>
+          <t>CC BY-SA 2.0</t>
+        </is>
+      </c>
       <c r="R8" s="23" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Boeing%2C_N8701Q%2C_Boeing_737-8_MAX_%282%29.jpg</t>
@@ -29832,9 +29916,21 @@
         </is>
       </c>
       <c r="N9" s="25" t="n"/>
-      <c r="O9" s="25" t="n"/>
-      <c r="P9" s="25" t="n"/>
-      <c r="Q9" s="25" t="n"/>
+      <c r="O9" s="25" t="inlineStr">
+        <is>
+          <t>b787.jpg</t>
+        </is>
+      </c>
+      <c r="P9" s="25" t="inlineStr">
+        <is>
+          <t>Maksim Sidorov</t>
+        </is>
+      </c>
+      <c r="Q9" s="25" t="inlineStr">
+        <is>
+          <t>CC BY 3.0</t>
+        </is>
+      </c>
       <c r="R9" s="25" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:N787BA_01.jpg</t>
@@ -29893,9 +29989,21 @@
         </is>
       </c>
       <c r="N10" s="25" t="n"/>
-      <c r="O10" s="25" t="n"/>
-      <c r="P10" s="25" t="n"/>
-      <c r="Q10" s="25" t="n"/>
+      <c r="O10" s="25" t="inlineStr">
+        <is>
+          <t>a350.jpg</t>
+        </is>
+      </c>
+      <c r="P10" s="25" t="inlineStr">
+        <is>
+          <t>Gyrostat</t>
+        </is>
+      </c>
+      <c r="Q10" s="25" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0</t>
+        </is>
+      </c>
       <c r="R10" s="25" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:AIB_A350_F-WXWB_24oct14_LFBO-2.jpg</t>
@@ -29954,9 +30062,21 @@
         </is>
       </c>
       <c r="N11" s="25" t="n"/>
-      <c r="O11" s="25" t="n"/>
-      <c r="P11" s="25" t="n"/>
-      <c r="Q11" s="25" t="n"/>
+      <c r="O11" s="25" t="inlineStr">
+        <is>
+          <t>b747.jpg</t>
+        </is>
+      </c>
+      <c r="P11" s="25" t="inlineStr">
+        <is>
+          <t>Boeing Dreamscape</t>
+        </is>
+      </c>
+      <c r="Q11" s="25" t="inlineStr">
+        <is>
+          <t>CC BY 2.0</t>
+        </is>
+      </c>
       <c r="R11" s="25" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Boeing_747-8_first_flight_Everett%2C_WA.jpg</t>
@@ -30015,9 +30135,21 @@
         </is>
       </c>
       <c r="N12" s="25" t="n"/>
-      <c r="O12" s="25" t="n"/>
-      <c r="P12" s="25" t="n"/>
-      <c r="Q12" s="25" t="n"/>
+      <c r="O12" s="25" t="inlineStr">
+        <is>
+          <t>a380.jpg</t>
+        </is>
+      </c>
+      <c r="P12" s="25" t="inlineStr">
+        <is>
+          <t>Anna Zvereva</t>
+        </is>
+      </c>
+      <c r="Q12" s="25" t="inlineStr">
+        <is>
+          <t>CC BY-SA 2.0</t>
+        </is>
+      </c>
       <c r="R12" s="25" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Airbus_Industrie%2C_F-WWOW%2C_Airbus_A380-841_%2835679929105%29.jpg</t>
@@ -30138,9 +30270,21 @@
           <t>e175</t>
         </is>
       </c>
-      <c r="O15" s="23" t="n"/>
-      <c r="P15" s="23" t="n"/>
-      <c r="Q15" s="23" t="n"/>
+      <c r="O15" s="23" t="inlineStr">
+        <is>
+          <t>e175.jpg</t>
+        </is>
+      </c>
+      <c r="P15" s="23" t="inlineStr">
+        <is>
+          <t>AVA Navigate</t>
+        </is>
+      </c>
+      <c r="Q15" s="23" t="inlineStr">
+        <is>
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
       <c r="R15" s="23" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Republic_Airways_N401YX_E75L.jpg</t>
@@ -30199,9 +30343,21 @@
         </is>
       </c>
       <c r="N16" s="27" t="n"/>
-      <c r="O16" s="27" t="n"/>
-      <c r="P16" s="27" t="n"/>
-      <c r="Q16" s="27" t="n"/>
+      <c r="O16" s="27" t="inlineStr">
+        <is>
+          <t>b757.jpg</t>
+        </is>
+      </c>
+      <c r="P16" s="27" t="inlineStr">
+        <is>
+          <t>Aeroprints.com</t>
+        </is>
+      </c>
+      <c r="Q16" s="27" t="inlineStr">
+        <is>
+          <t>CC BY-SA 3.0</t>
+        </is>
+      </c>
       <c r="R16" s="27" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:N767AN_Boeing_757F_All_White_Colours_%288736741972%29.jpg</t>
@@ -30260,9 +30416,21 @@
         </is>
       </c>
       <c r="N17" s="25" t="n"/>
-      <c r="O17" s="25" t="n"/>
-      <c r="P17" s="25" t="n"/>
-      <c r="Q17" s="25" t="n"/>
+      <c r="O17" s="25" t="inlineStr">
+        <is>
+          <t>a340.jpg</t>
+        </is>
+      </c>
+      <c r="P17" s="25" t="inlineStr">
+        <is>
+          <t>Ken Fielding</t>
+        </is>
+      </c>
+      <c r="Q17" s="25" t="inlineStr">
+        <is>
+          <t>CC BY-SA 3.0</t>
+        </is>
+      </c>
       <c r="R17" s="25" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:F-WWCA_A340-642_%28proto%29_Airbus_TLS_09SEP10_%284979496505%29.jpg</t>
@@ -30321,9 +30489,21 @@
         </is>
       </c>
       <c r="N18" s="25" t="n"/>
-      <c r="O18" s="25" t="n"/>
-      <c r="P18" s="25" t="n"/>
-      <c r="Q18" s="25" t="n"/>
+      <c r="O18" s="25" t="inlineStr">
+        <is>
+          <t>b777.jpg</t>
+        </is>
+      </c>
+      <c r="P18" s="25" t="inlineStr">
+        <is>
+          <t>Mztourist</t>
+        </is>
+      </c>
+      <c r="Q18" s="25" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0</t>
+        </is>
+      </c>
       <c r="R18" s="25" t="inlineStr">
         <is>
           <t>https://commons.wikimedia.org/wiki/File:Boeing_777X_at_Dubai_Airshow_2021_3.jpg</t>

</xml_diff>

<commit_message>
Workbook v4.4 data and rules (stage A): play mode, day costs and prices, Buy greyed until affordable, use-it-or-lose-it, best-plan sweep
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013x87PezhtynWHJHngTWCer
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -696,14 +696,21 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>v4.3 + CR5 rows re-added by Claude Code (8 Oct): Fable's v4.3 did not carry the CR5 draft, so the Livery sheet, the Aircraft columns artworkId/photoFile/photoCredit/photoLicence/photoSource, and Settings blockedFlightCodes, soundDefault, revealSeconds are added again, plus practiceQuestionsPerDay (design note). The game reads crewMechanicFromDate (D51); the earlier draft key crewFromDate is dropped.</t>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>v4.4 (12 Oct): D52–D55. Chapter 1 is played a WEEK at a time (Calendar weekPhase: plan / run / review; days 1–28 rewritten); both routes from Launch Day; week 2 = second plane; four routes week 3; Madrid week 4; Marrakech and weekly skips from day 29; later routes and the A220/A320/737 shift a week. Tutorial plane prices 2½× (second plane rented or financed first); aircraft day costs raised (bad plans lose money); missed-profit line in every weekly review; use-it-or-lose-it from week 3 (Settings neglect*). Chapter-1 events aligned to Mondays. Balance Report v4.4 addendum.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>v4.3 + CR5 rows re-added by Claude Code (8 Oct): Fable's v4.3 did not carry the CR5 draft, so the Livery sheet, the Aircraft columns artworkId/photoFile/photoCredit/photoLicence/photoSource, and Settings blockedFlightCodes, soundDefault, revealSeconds are added again, plus practiceQuestionsPerDay (design note). The game reads crewMechanicFromDate (D51); the earlier draft key crewFromDate is dropped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>v4.3 draft (7 Oct, Claude Code, for Fable to adopt): Change Request 5. New sheet Livery (palette, stripes, tail symbols, logo shapes, plane-name suggestions); Aircraft columns artworkId and photoFile/Credit/Licence/Source; Settings blockedFlightCodes, soundDefault, revealSeconds. Everything the pupil chooses (airline name, flight code, logo, each plane's registration, name and livery) lives in the save state, not here.</t>
         </is>
@@ -1028,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q22"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1136,951 +1143,927 @@
           <t>status</t>
         </is>
       </c>
+      <c r="R1" s="20" t="inlineStr">
+        <is>
+          <t>weekPhase</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="A2" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>2030-09-02</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="D2" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="12" t="inlineStr">
-        <is>
-          <t>setup</t>
-        </is>
-      </c>
-      <c r="F2" s="12" t="n">
+      <c r="D2" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="n">
         <v>1.2</v>
       </c>
-      <c r="G2" s="12" t="inlineStr">
-        <is>
-          <t>Launch day</t>
-        </is>
-      </c>
-      <c r="H2" s="12" t="inlineStr">
-        <is>
-          <t>New airline launches from London.</t>
-        </is>
-      </c>
-      <c r="I2" s="12" t="inlineStr">
-        <is>
-          <t>Fuel steady at £1.20 a litre.</t>
-        </is>
-      </c>
-      <c r="J2" s="12" t="inlineStr"/>
-      <c r="K2" s="12" t="inlineStr">
-        <is>
-          <t>routes: first market (pupil chooses dub or par); planes: dhc6 (launch deal); mechanics: fare, services, timetable</t>
-        </is>
-      </c>
-      <c r="L2" s="12" t="inlineStr"/>
-      <c r="M2" s="12" t="inlineStr"/>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Launch Day: build your standing plan</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>Your airline is cleared for take-off. Build the week's plan: timetable, fare, snacks, fuel.</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="inlineStr">
+        <is>
+          <t>Fuel is free today and tomorrow.</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr"/>
+      <c r="K2" s="13" t="inlineStr">
+        <is>
+          <t>routes: dub, par; planes: dhc6 (launch deal); mechanics: timetable with demand curve, fare, snacks, fuel, modelling tool, workings page</t>
+        </is>
+      </c>
+      <c r="L2" s="13" t="inlineStr"/>
+      <c r="M2" s="13" t="n"/>
+      <c r="N2" s="13" t="inlineStr">
+        <is>
+          <t>pricing,timetable,cabin,fuel</t>
+        </is>
+      </c>
+      <c r="O2" s="13" t="inlineStr">
+        <is>
+          <t>ticketRevenue,profit,snackRevenue,fuelCost</t>
+        </is>
+      </c>
+      <c r="P2" s="13" t="n"/>
+      <c r="Q2" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R2" s="13" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-03</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Day two runs to plan.</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>Fuel is free today.</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr"/>
+      <c r="K3" s="13" t="inlineStr"/>
+      <c r="L3" s="13" t="inlineStr"/>
+      <c r="M3" s="13" t="n"/>
+      <c r="N3" s="13" t="inlineStr"/>
+      <c r="O3" s="13" t="inlineStr"/>
+      <c r="P3" s="13" t="n"/>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R3" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-04</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Wednesday: fuel is yours to buy</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>The launch deal is over: from today you buy your own fuel.</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Fuel £1.30 a litre.</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr"/>
+      <c r="K4" s="13" t="inlineStr"/>
+      <c r="L4" s="13" t="inlineStr"/>
+      <c r="M4" s="13" t="n"/>
+      <c r="N4" s="13" t="inlineStr"/>
+      <c r="O4" s="13" t="inlineStr"/>
+      <c r="P4" s="13" t="n"/>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R4" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-05</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Thursday: Red Kite</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Red Kite Air is selling Dublin at £50 until Sunday.</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr"/>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>undercut_dub</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr"/>
+      <c r="L5" s="13" t="inlineStr"/>
+      <c r="M5" s="13" t="n"/>
+      <c r="N5" s="13" t="inlineStr">
         <is>
           <t>pricing</t>
         </is>
       </c>
-      <c r="O2" s="12" t="inlineStr">
-        <is>
-          <t>revenue</t>
-        </is>
-      </c>
-      <c r="P2" s="12" t="inlineStr"/>
-      <c r="Q2" s="12" t="inlineStr">
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>rivalSwitch</t>
+        </is>
+      </c>
+      <c r="P5" s="13" t="n"/>
+      <c r="Q5" s="13" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="12" t="n">
+      <c r="R5" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-06</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>Friday: storm</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>A storm is forecast for this afternoon.</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>Fuel £1.40 a litre.</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>storm</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr"/>
+      <c r="M6" s="13" t="n"/>
+      <c r="N6" s="13" t="inlineStr"/>
+      <c r="O6" s="13" t="inlineStr"/>
+      <c r="P6" s="13" t="n"/>
+      <c r="Q6" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R6" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-07</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>Quiet at the airport: business travellers stay home, families fly.</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr"/>
+      <c r="J7" s="13" t="inlineStr"/>
+      <c r="K7" s="13" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>weekend multipliers (Settings)</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="n"/>
+      <c r="N7" s="13" t="inlineStr"/>
+      <c r="O7" s="13" t="inlineStr"/>
+      <c r="P7" s="13" t="n"/>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R7" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-08</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Sunday: the week's accounts</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>Seven days flown. Add up the week; compare it with the plan.</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="inlineStr"/>
+      <c r="J8" s="13" t="inlineStr"/>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>mechanics: weekly review, seven-row table, projected − actual, missed-profit line</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>weekend multipliers (Settings)</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="n"/>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>weekTotal,projectedVsActual</t>
+        </is>
+      </c>
+      <c r="P8" s="13" t="n"/>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R8" s="13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-09</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-03</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Week 2: a second plane</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>One plane cannot serve both routes fully. The shop has a Saab 340 and an ATR 72. Rent, finance, or save to buy?</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>Fuel £1.50 a litre.</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr"/>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>planes: dhc6 (second), saab340, atr72; mechanics: rent-or-buy sum, launch-deal finance, buy greyed until affordable, two timetables, assignment</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr"/>
+      <c r="M9" s="13" t="n"/>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>fleet,assignment,timetable</t>
+        </is>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>rentOrBuy</t>
+        </is>
+      </c>
+      <c r="P9" s="13" t="n"/>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R9" s="13" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-10</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D3" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="D10" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="F3" s="12" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>A catering offer</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>A catering supplier offers snacks on board.</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>Fuel steady at £1.20 a litre.</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="inlineStr"/>
-      <c r="K3" s="12" t="inlineStr">
-        <is>
-          <t>mechanics: snacks (on-board sales)</t>
-        </is>
-      </c>
-      <c r="L3" s="12" t="inlineStr"/>
-      <c r="M3" s="12" t="inlineStr"/>
-      <c r="N3" s="12" t="inlineStr">
-        <is>
-          <t>pricing,cabin</t>
-        </is>
-      </c>
-      <c r="O3" s="12" t="inlineStr">
-        <is>
-          <t>snackRevenue</t>
-        </is>
-      </c>
-      <c r="P3" s="12" t="inlineStr"/>
-      <c r="Q3" s="12" t="inlineStr">
+      <c r="F10" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Two planes on the board.</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="inlineStr"/>
+      <c r="J10" s="13" t="inlineStr"/>
+      <c r="K10" s="13" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr"/>
+      <c r="M10" s="13" t="n"/>
+      <c r="N10" s="13" t="inlineStr"/>
+      <c r="O10" s="13" t="inlineStr"/>
+      <c r="P10" s="13" t="n"/>
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="R10" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-11</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>Fuel £1.60 a litre.</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr"/>
+      <c r="K11" s="13" t="inlineStr"/>
+      <c r="L11" s="13" t="inlineStr"/>
+      <c r="M11" s="13" t="n"/>
+      <c r="N11" s="13" t="inlineStr"/>
+      <c r="O11" s="13" t="inlineStr"/>
+      <c r="P11" s="13" t="n"/>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R11" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-12</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Thursday: crew sickness</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>The captain has flu.</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="inlineStr"/>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>crew</t>
+        </is>
+      </c>
+      <c r="K12" s="13" t="inlineStr"/>
+      <c r="L12" s="13" t="inlineStr"/>
+      <c r="M12" s="13" t="n"/>
+      <c r="N12" s="13" t="inlineStr"/>
+      <c r="O12" s="13" t="inlineStr"/>
+      <c r="P12" s="13" t="n"/>
+      <c r="Q12" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R12" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-13</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>Fuel £1.70 a litre.</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr"/>
+      <c r="K13" s="13" t="inlineStr"/>
+      <c r="L13" s="13" t="inlineStr"/>
+      <c r="M13" s="13" t="n"/>
+      <c r="N13" s="13" t="inlineStr"/>
+      <c r="O13" s="13" t="inlineStr"/>
+      <c r="P13" s="13" t="n"/>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R13" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-14</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr"/>
+      <c r="I14" s="13" t="inlineStr"/>
+      <c r="J14" s="13" t="inlineStr"/>
+      <c r="K14" s="13" t="inlineStr"/>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>weekend multipliers (Settings)</t>
+        </is>
+      </c>
+      <c r="M14" s="13" t="n"/>
+      <c r="N14" s="13" t="inlineStr"/>
+      <c r="O14" s="13" t="inlineStr"/>
+      <c r="P14" s="13" t="n"/>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R14" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-15</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Sunday: week 2 accounts</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr"/>
+      <c r="I15" s="13" t="inlineStr"/>
+      <c r="J15" s="13" t="inlineStr"/>
+      <c r="K15" s="13" t="inlineStr"/>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>weekend multipliers (Settings)</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="n"/>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>weekTotal,projectedVsActual</t>
+        </is>
+      </c>
+      <c r="P15" s="13" t="n"/>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R15" s="13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-16</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-04</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="F4" s="12" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>Fuel on the move</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>Fuel rises to £1.30 a litre.</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>Oil experts say fuel will keep rising this year.</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="inlineStr"/>
-      <c r="K4" s="12" t="inlineStr">
-        <is>
-          <t>mechanics:fuel,tank</t>
-        </is>
-      </c>
-      <c r="L4" s="12" t="inlineStr"/>
-      <c r="M4" s="12" t="inlineStr"/>
-      <c r="N4" s="12" t="inlineStr">
-        <is>
-          <t>fuel,pricing</t>
-        </is>
-      </c>
-      <c r="O4" s="12" t="inlineStr">
-        <is>
-          <t>fuel</t>
-        </is>
-      </c>
-      <c r="P4" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="12" t="inlineStr">
+      <c r="F16" s="13" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>Week 3: four new routes</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>Amsterdam, Frankfurt, Geneva and Barcelona open. Fares step by £5.</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>Fuel £1.70 a litre. Red Kite flies from Luton.</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>routes: ams, fra, gva, bcn; mechanics: £5 fares, season badge on route cards, use-it-or-lose-it from this week</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr"/>
+      <c r="M16" s="13" t="n"/>
+      <c r="N16" s="13" t="inlineStr">
+        <is>
+          <t>pricing,assignment,timetable</t>
+        </is>
+      </c>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t>ticketRevenueLong,flightTime</t>
+        </is>
+      </c>
+      <c r="P16" s="13" t="n"/>
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-05</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>Red Kite arrives</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>Red Kite Air cuts Dublin fares to £50!</t>
-        </is>
-      </c>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>Fuel £1.30 a litre.</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>undercut_dub</t>
-        </is>
-      </c>
-      <c r="K5" s="12" t="inlineStr">
-        <is>
-          <t>routes: the other of dub/par; mechanics: rival fares, time-of-day demand, second route</t>
-        </is>
-      </c>
-      <c r="L5" s="12" t="inlineStr"/>
-      <c r="M5" s="12" t="inlineStr">
-        <is>
-          <t>dub:50</t>
-        </is>
-      </c>
-      <c r="N5" s="12" t="inlineStr">
-        <is>
-          <t>pricing</t>
-        </is>
-      </c>
-      <c r="O5" s="12" t="inlineStr">
-        <is>
-          <t>revenue</t>
-        </is>
-      </c>
-      <c r="P5" s="12" t="inlineStr"/>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-06</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>The storm</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>Storm warning: strong winds over the Irish Sea.</t>
-        </is>
-      </c>
-      <c r="I6" s="12" t="inlineStr">
-        <is>
-          <t>Fuel £1.40 a litre and rising.</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="inlineStr">
-        <is>
-          <t>storm</t>
-        </is>
-      </c>
-      <c r="K6" s="12" t="inlineStr">
-        <is>
-          <t>mechanics:crew duty</t>
-        </is>
-      </c>
-      <c r="L6" s="12" t="inlineStr"/>
-      <c r="M6" s="12" t="inlineStr">
-        <is>
-          <t>dub:50</t>
-        </is>
-      </c>
-      <c r="N6" s="12" t="inlineStr">
-        <is>
-          <t>checkFlight,pricing</t>
-        </is>
-      </c>
-      <c r="O6" s="12" t="inlineStr">
-        <is>
-          <t>flight</t>
-        </is>
-      </c>
-      <c r="P6" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-07</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>weekend</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
-        <is>
-          <t>Quiet weekend at the airport. Business travellers stay home; families fly.</t>
-        </is>
-      </c>
-      <c r="I7" s="12" t="inlineStr"/>
-      <c r="J7" s="12" t="inlineStr"/>
-      <c r="K7" s="12" t="inlineStr"/>
-      <c r="L7" s="12" t="inlineStr">
-        <is>
-          <t>weekend multipliers (Settings)</t>
-        </is>
-      </c>
-      <c r="M7" s="12" t="inlineStr">
-        <is>
-          <t>dub:50</t>
-        </is>
-      </c>
-      <c r="N7" s="12" t="inlineStr"/>
-      <c r="O7" s="12" t="inlineStr"/>
-      <c r="P7" s="12" t="inlineStr"/>
-      <c r="Q7" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-08</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>weekend</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="inlineStr"/>
-      <c r="I8" s="12" t="inlineStr"/>
-      <c r="J8" s="12" t="inlineStr"/>
-      <c r="K8" s="12" t="inlineStr"/>
-      <c r="L8" s="12" t="inlineStr">
-        <is>
-          <t>weekend multipliers (Settings)</t>
-        </is>
-      </c>
-      <c r="M8" s="12" t="inlineStr">
-        <is>
-          <t>dub:50</t>
-        </is>
-      </c>
-      <c r="N8" s="12" t="inlineStr"/>
-      <c r="O8" s="12" t="inlineStr"/>
-      <c r="P8" s="12" t="inlineStr"/>
-      <c r="Q8" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-09</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>Week 2: a bigger airline</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr">
-        <is>
-          <t>Four new destinations open. Time to choose a second aircraft.</t>
-        </is>
-      </c>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>Fuel £1.50 a litre. Red Kite, flying from Luton, says its costs are lower than yours.</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="inlineStr"/>
-      <c r="K9" s="12" t="inlineStr">
-        <is>
-          <t>routes:ams,fra,gva,bcn; planes:saab340,atr72,dhc6; mechanics:assignment,finance,season badge</t>
-        </is>
-      </c>
-      <c r="L9" s="12" t="inlineStr"/>
-      <c r="M9" s="12" t="inlineStr"/>
-      <c r="N9" s="12" t="inlineStr">
-        <is>
-          <t>fleet,assignment,pricing</t>
-        </is>
-      </c>
-      <c r="O9" s="12" t="inlineStr">
-        <is>
-          <t>revenue</t>
-        </is>
-      </c>
-      <c r="P9" s="12" t="inlineStr"/>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-10</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>Two planes, two plans</t>
-        </is>
-      </c>
-      <c r="H10" s="12" t="inlineStr">
-        <is>
-          <t>Your second aircraft flies today.</t>
-        </is>
-      </c>
-      <c r="I10" s="12" t="inlineStr">
-        <is>
-          <t>Barcelona still warm; Geneva quiet until the snow.</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="inlineStr"/>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>mechanics:two timetables</t>
-        </is>
-      </c>
-      <c r="L10" s="12" t="inlineStr"/>
-      <c r="M10" s="12" t="inlineStr"/>
-      <c r="N10" s="12" t="inlineStr">
-        <is>
-          <t>assignment,pricing</t>
-        </is>
-      </c>
-      <c r="O10" s="12" t="inlineStr">
-        <is>
-          <t>revenue</t>
-        </is>
-      </c>
-      <c r="P10" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-11</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>Who flies where?</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>Amsterdam is heaving. Paris is not.</t>
-        </is>
-      </c>
-      <c r="I11" s="12" t="inlineStr">
-        <is>
-          <t>Fuel £1.60 a litre.</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="inlineStr"/>
-      <c r="K11" s="12" t="inlineStr"/>
-      <c r="L11" s="12" t="inlineStr"/>
-      <c r="M11" s="12" t="inlineStr"/>
-      <c r="N11" s="12" t="inlineStr">
-        <is>
-          <t>assignment,fuel</t>
-        </is>
-      </c>
-      <c r="O11" s="12" t="inlineStr">
-        <is>
-          <t>fuel</t>
-        </is>
-      </c>
-      <c r="P11" s="12" t="inlineStr"/>
-      <c r="Q11" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-12</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>Crew sickness</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr">
-        <is>
-          <t>Flu going round the airport this week.</t>
-        </is>
-      </c>
-      <c r="I12" s="12" t="inlineStr">
-        <is>
-          <t>Fuel £1.60 a litre.</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="inlineStr">
-        <is>
-          <t>crew</t>
-        </is>
-      </c>
-      <c r="K12" s="12" t="inlineStr"/>
-      <c r="L12" s="12" t="inlineStr"/>
-      <c r="M12" s="12" t="inlineStr"/>
-      <c r="N12" s="12" t="inlineStr">
-        <is>
-          <t>pricing</t>
-        </is>
-      </c>
-      <c r="O12" s="12" t="inlineStr">
-        <is>
-          <t>revenue</t>
-        </is>
-      </c>
-      <c r="P12" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q12" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-13</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>Season forecast</t>
-        </is>
-      </c>
-      <c r="H13" s="12" t="inlineStr">
-        <is>
-          <t>Weather office: a cold, snowy winter is on the way.</t>
-        </is>
-      </c>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>Fuel £1.70 a litre.</t>
-        </is>
-      </c>
-      <c r="J13" s="12" t="inlineStr"/>
-      <c r="K13" s="12" t="inlineStr">
-        <is>
-          <t>mechanics:season forecast card</t>
-        </is>
-      </c>
-      <c r="L13" s="12" t="inlineStr">
-        <is>
-          <t>gva:+10</t>
-        </is>
-      </c>
-      <c r="M13" s="12" t="inlineStr"/>
-      <c r="N13" s="12" t="inlineStr">
-        <is>
-          <t>pricing,cabin</t>
-        </is>
-      </c>
-      <c r="O13" s="12" t="inlineStr">
-        <is>
-          <t>cabin</t>
-        </is>
-      </c>
-      <c r="P13" s="12" t="inlineStr"/>
-      <c r="Q13" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-14</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>weekend</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="H14" s="12" t="inlineStr"/>
-      <c r="I14" s="12" t="inlineStr"/>
-      <c r="J14" s="12" t="inlineStr"/>
-      <c r="K14" s="12" t="inlineStr"/>
-      <c r="L14" s="12" t="inlineStr">
-        <is>
-          <t>weekend multipliers (Settings)</t>
-        </is>
-      </c>
-      <c r="M14" s="12" t="inlineStr"/>
-      <c r="N14" s="12" t="inlineStr"/>
-      <c r="O14" s="12" t="inlineStr"/>
-      <c r="P14" s="12" t="inlineStr"/>
-      <c r="Q14" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-15</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>weekend</t>
-        </is>
-      </c>
-      <c r="F15" s="12" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="H15" s="12" t="inlineStr"/>
-      <c r="I15" s="12" t="inlineStr"/>
-      <c r="J15" s="12" t="inlineStr"/>
-      <c r="K15" s="12" t="inlineStr"/>
-      <c r="L15" s="12" t="inlineStr">
-        <is>
-          <t>weekend multipliers (Settings)</t>
-        </is>
-      </c>
-      <c r="M15" s="12" t="inlineStr"/>
-      <c r="N15" s="12" t="inlineStr"/>
-      <c r="O15" s="12" t="inlineStr"/>
-      <c r="P15" s="12" t="inlineStr"/>
-      <c r="Q15" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>2030-09-16</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>Week 3: medium haul</t>
-        </is>
-      </c>
-      <c r="H16" s="12" t="inlineStr">
-        <is>
-          <t>Madrid opens. A jet appears in the shop.</t>
-        </is>
-      </c>
-      <c r="I16" s="12" t="inlineStr">
-        <is>
-          <t>Fuel £1.70 a litre.</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="inlineStr"/>
-      <c r="K16" s="12" t="inlineStr">
-        <is>
-          <t>routes: mad; planes: e190; mechanics: range check, services per day on a long leg (ATR or E190)</t>
-        </is>
-      </c>
-      <c r="L16" s="12" t="inlineStr"/>
-      <c r="M16" s="12" t="inlineStr"/>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>fleet,assignment,pricing</t>
-        </is>
-      </c>
-      <c r="O16" s="12" t="inlineStr">
-        <is>
-          <t>range,flightTime</t>
-        </is>
-      </c>
-      <c r="P16" s="12" t="inlineStr"/>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="R16" s="13" t="inlineStr">
+        <is>
+          <t>plan</t>
         </is>
       </c>
     </row>
@@ -2111,33 +2094,26 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>Two planes, three routes</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>Where does the jet earn most?</t>
-        </is>
-      </c>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr"/>
       <c r="I17" s="13" t="inlineStr"/>
-      <c r="J17" s="13" t="n"/>
-      <c r="K17" s="13" t="n"/>
+      <c r="J17" s="13" t="inlineStr"/>
+      <c r="K17" s="13" t="inlineStr"/>
       <c r="L17" s="13" t="inlineStr"/>
       <c r="M17" s="13" t="n"/>
-      <c r="N17" s="13" t="inlineStr">
-        <is>
-          <t>assignment,pricing</t>
-        </is>
-      </c>
-      <c r="O17" s="13" t="inlineStr">
-        <is>
-          <t>revenue</t>
-        </is>
-      </c>
+      <c r="N17" s="13" t="inlineStr"/>
+      <c r="O17" s="13" t="inlineStr"/>
       <c r="P17" s="13" t="n"/>
       <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>live</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
         </is>
       </c>
     </row>
@@ -2168,37 +2144,26 @@
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>Fuel for a jet</t>
-        </is>
-      </c>
-      <c r="H18" s="13" t="inlineStr">
-        <is>
-          <t>A jet burns in one trip what a Twin Otter burns in a week.</t>
-        </is>
-      </c>
-      <c r="I18" s="13" t="inlineStr">
-        <is>
-          <t>Fuel £1.70 a litre.</t>
-        </is>
-      </c>
-      <c r="J18" s="13" t="n"/>
-      <c r="K18" s="13" t="n"/>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr"/>
+      <c r="I18" s="13" t="inlineStr"/>
+      <c r="J18" s="13" t="inlineStr"/>
+      <c r="K18" s="13" t="inlineStr"/>
       <c r="L18" s="13" t="inlineStr"/>
       <c r="M18" s="13" t="n"/>
-      <c r="N18" s="13" t="inlineStr">
-        <is>
-          <t>fuel</t>
-        </is>
-      </c>
-      <c r="O18" s="13" t="inlineStr">
-        <is>
-          <t>fuel</t>
-        </is>
-      </c>
+      <c r="N18" s="13" t="inlineStr"/>
+      <c r="O18" s="13" t="inlineStr"/>
       <c r="P18" s="13" t="n"/>
       <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>live</t>
+        </is>
+      </c>
+      <c r="R18" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
         </is>
       </c>
     </row>
@@ -2229,33 +2194,26 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>Red Kite copies you</t>
-        </is>
-      </c>
-      <c r="H19" s="13" t="inlineStr">
-        <is>
-          <t>Red Kite announces Madrid flights from Luton.</t>
-        </is>
-      </c>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr"/>
       <c r="I19" s="13" t="inlineStr"/>
-      <c r="J19" s="13" t="n"/>
-      <c r="K19" s="13" t="n"/>
+      <c r="J19" s="13" t="inlineStr"/>
+      <c r="K19" s="13" t="inlineStr"/>
       <c r="L19" s="13" t="inlineStr"/>
       <c r="M19" s="13" t="n"/>
-      <c r="N19" s="13" t="inlineStr">
-        <is>
-          <t>pricing</t>
-        </is>
-      </c>
-      <c r="O19" s="13" t="inlineStr">
-        <is>
-          <t>revenue</t>
-        </is>
-      </c>
+      <c r="N19" s="13" t="inlineStr"/>
+      <c r="O19" s="13" t="inlineStr"/>
       <c r="P19" s="13" t="n"/>
       <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>live</t>
+        </is>
+      </c>
+      <c r="R19" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
         </is>
       </c>
     </row>
@@ -2286,33 +2244,34 @@
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>Full planes</t>
+          <t>Friday: the season forecast</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Operations: the Madrid flight was full. Was the fare right?</t>
+          <t>The weather office forecasts a cold, snowy winter.</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
+      <c r="J20" s="13" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>mechanics: season forecast card</t>
+        </is>
+      </c>
       <c r="L20" s="13" t="inlineStr"/>
       <c r="M20" s="13" t="n"/>
-      <c r="N20" s="13" t="inlineStr">
-        <is>
-          <t>pricing</t>
-        </is>
-      </c>
-      <c r="O20" s="13" t="inlineStr">
-        <is>
-          <t>emptySeats</t>
-        </is>
-      </c>
+      <c r="N20" s="13" t="inlineStr"/>
+      <c r="O20" s="13" t="inlineStr"/>
       <c r="P20" s="13" t="n"/>
       <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>live</t>
+        </is>
+      </c>
+      <c r="R20" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
         </is>
       </c>
     </row>
@@ -2348,8 +2307,8 @@
       </c>
       <c r="H21" s="13" t="inlineStr"/>
       <c r="I21" s="13" t="inlineStr"/>
-      <c r="J21" s="13" t="n"/>
-      <c r="K21" s="13" t="n"/>
+      <c r="J21" s="13" t="inlineStr"/>
+      <c r="K21" s="13" t="inlineStr"/>
       <c r="L21" s="13" t="inlineStr">
         <is>
           <t>weekend multipliers (Settings)</t>
@@ -2364,6 +2323,11 @@
           <t>live</t>
         </is>
       </c>
+      <c r="R21" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="n">
@@ -2392,25 +2356,448 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Sunday: week 3 accounts</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr"/>
       <c r="I22" s="13" t="inlineStr"/>
-      <c r="J22" s="13" t="n"/>
-      <c r="K22" s="13" t="n"/>
+      <c r="J22" s="13" t="inlineStr"/>
+      <c r="K22" s="13" t="inlineStr"/>
       <c r="L22" s="13" t="inlineStr">
         <is>
           <t>weekend multipliers (Settings)</t>
         </is>
       </c>
       <c r="M22" s="13" t="n"/>
-      <c r="N22" s="13" t="inlineStr"/>
-      <c r="O22" s="13" t="inlineStr"/>
+      <c r="N22" s="13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="O22" s="13" t="inlineStr">
+        <is>
+          <t>weekTotal,projectedVsActual</t>
+        </is>
+      </c>
       <c r="P22" s="13" t="n"/>
       <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>live</t>
+        </is>
+      </c>
+      <c r="R22" s="13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-23</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>Week 4: medium haul</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>Madrid opens. Two jets are in the shop: the E175 and the E190. Does your plane have the range?</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>Fuel £1.80 a litre.</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr"/>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>routes: mad; planes: e175, e190; mechanics: range check, services per day on a long leg, load factor as a percentage</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="inlineStr"/>
+      <c r="M23" s="13" t="n"/>
+      <c r="N23" s="13" t="inlineStr">
+        <is>
+          <t>fleet,assignment,pricing</t>
+        </is>
+      </c>
+      <c r="O23" s="13" t="inlineStr">
+        <is>
+          <t>range,flightTime,loadFactor</t>
+        </is>
+      </c>
+      <c r="P23" s="13" t="n"/>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R23" s="13" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-24</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr"/>
+      <c r="I24" s="13" t="inlineStr"/>
+      <c r="J24" s="13" t="inlineStr"/>
+      <c r="K24" s="13" t="inlineStr"/>
+      <c r="L24" s="13" t="inlineStr"/>
+      <c r="M24" s="13" t="n"/>
+      <c r="N24" s="13" t="inlineStr"/>
+      <c r="O24" s="13" t="inlineStr"/>
+      <c r="P24" s="13" t="n"/>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R24" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-25</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>Wednesday: fuel for a jet</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>A jet burns in one trip what a Twin Otter burns in a week.</t>
+        </is>
+      </c>
+      <c r="I25" s="13" t="inlineStr"/>
+      <c r="J25" s="13" t="inlineStr"/>
+      <c r="K25" s="13" t="inlineStr"/>
+      <c r="L25" s="13" t="inlineStr"/>
+      <c r="M25" s="13" t="n"/>
+      <c r="N25" s="13" t="inlineStr">
+        <is>
+          <t>fuel</t>
+        </is>
+      </c>
+      <c r="O25" s="13" t="inlineStr">
+        <is>
+          <t>fuelCost</t>
+        </is>
+      </c>
+      <c r="P25" s="13" t="n"/>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R25" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-26</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>Thursday: Red Kite copies you</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>Red Kite announces Madrid flights from Luton.</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr"/>
+      <c r="J26" s="13" t="inlineStr"/>
+      <c r="K26" s="13" t="inlineStr"/>
+      <c r="L26" s="13" t="inlineStr"/>
+      <c r="M26" s="13" t="n"/>
+      <c r="N26" s="13" t="inlineStr"/>
+      <c r="O26" s="13" t="inlineStr"/>
+      <c r="P26" s="13" t="n"/>
+      <c r="Q26" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R26" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-27</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr"/>
+      <c r="J27" s="13" t="inlineStr"/>
+      <c r="K27" s="13" t="inlineStr"/>
+      <c r="L27" s="13" t="inlineStr"/>
+      <c r="M27" s="13" t="n"/>
+      <c r="N27" s="13" t="inlineStr"/>
+      <c r="O27" s="13" t="inlineStr"/>
+      <c r="P27" s="13" t="n"/>
+      <c r="Q27" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R27" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-28</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr"/>
+      <c r="I28" s="13" t="inlineStr"/>
+      <c r="J28" s="13" t="inlineStr"/>
+      <c r="K28" s="13" t="inlineStr"/>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>weekend multipliers (Settings)</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="n"/>
+      <c r="N28" s="13" t="inlineStr"/>
+      <c r="O28" s="13" t="inlineStr"/>
+      <c r="P28" s="13" t="n"/>
+      <c r="Q28" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R28" s="13" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>2030-09-29</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>Sunday: week 4 accounts; chapter 1 moves to weekly play</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>From next week the game runs a week at a time.</t>
+        </is>
+      </c>
+      <c r="I29" s="13" t="inlineStr"/>
+      <c r="J29" s="13" t="inlineStr"/>
+      <c r="K29" s="13" t="inlineStr">
+        <is>
+          <t>mechanics: weekly skips begin day 29</t>
+        </is>
+      </c>
+      <c r="L29" s="13" t="inlineStr">
+        <is>
+          <t>weekend multipliers (Settings)</t>
+        </is>
+      </c>
+      <c r="M29" s="13" t="n"/>
+      <c r="N29" s="13" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="O29" s="13" t="inlineStr">
+        <is>
+          <t>weekTotal,projectedVsActual</t>
+        </is>
+      </c>
+      <c r="P29" s="13" t="n"/>
+      <c r="Q29" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="R29" s="13" t="inlineStr">
+        <is>
+          <t>review</t>
         </is>
       </c>
     </row>
@@ -20340,7 +20727,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>2030-10-15</t>
+          <t>2030-10-14</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -20424,7 +20811,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>2030-11-03</t>
+          <t>2030-11-02</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -20464,7 +20851,7 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>2030-11-12</t>
+          <t>2030-11-11</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
@@ -20518,7 +20905,7 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>2030-12-03</t>
+          <t>2030-12-02</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -20558,7 +20945,7 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>2030-12-17</t>
+          <t>2030-12-16</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
@@ -21961,7 +22348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -21998,12 +22385,12 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>Fare, services, plane-loads, timetable</t>
+          <t>Launch Day: standing plan on one page; all opening sums in one sitting (tickets ×3, profit, snacks ×2, fuel); both routes; modelling tool; workings page</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Launch Day</t>
+          <t>D52, D54</t>
         </is>
       </c>
       <c r="D2" s="13" t="inlineStr">
@@ -22018,10 +22405,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Snacks (by hand once, then model)</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr"/>
+          <t>The week runs day by day on the operations board; results equal the projection; pauses for events (day 4 Red Kite with numbers, day 5 storm)</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>D52, D50</t>
+        </is>
+      </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
           <t>live</t>
@@ -22030,14 +22421,18 @@
     </row>
     <row r="4">
       <c r="A4" s="13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Fuel: litres, price, tank</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr"/>
+          <t>Weekly review every Sunday: seven-row table, total by hand, projected − actual, missed-profit line</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>D55</t>
+        </is>
+      </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
           <t>live</t>
@@ -22046,14 +22441,18 @@
     </row>
     <row r="5">
       <c r="A5" s="13" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Rival fares; time-of-day demand; second route</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr"/>
+          <t>Week 2: second plane; rent-or-buy sum; launch-deal finance; Buy greyed until affordable; two timetables; assignment</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>D53, D55</t>
+        </is>
+      </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
           <t>live</t>
@@ -22062,14 +22461,18 @@
     </row>
     <row r="6">
       <c r="A6" s="13" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Crew duty and second crew</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr"/>
+          <t>Week 3: four routes; £5 fares; season badge; use-it-or-lose-it begins</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>D28, D55</t>
+        </is>
+      </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
           <t>live</t>
@@ -22078,11 +22481,11 @@
     </row>
     <row r="7">
       <c r="A7" s="13" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Weekend demand</t>
+          <t>Season forecast card</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr"/>
@@ -22094,16 +22497,16 @@
     </row>
     <row r="8">
       <c r="A8" s="13" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Second plane: buy or rent (tutorial tier); the rent-or-buy sum; assignment; season badge; £5 fares</t>
+          <t>Week 4: medium haul; range check; services per day; E175 and E190; load factor as a percentage</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Week 2</t>
+          <t>D19, D23</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -22114,14 +22517,18 @@
     </row>
     <row r="9">
       <c r="A9" s="13" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Two timetables; one plane on two routes</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr"/>
+          <t>Week-at-a-time skips; Marrakech; event costs as a share of a day</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
           <t>live</t>
@@ -22129,12 +22536,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="n">
-        <v>12</v>
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>2030-12-02</t>
+        </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Season forecast card</t>
+          <t>Month-at-a-time play; monthly reports from here on</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr"/>
@@ -22145,19 +22554,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="n">
-        <v>15</v>
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>2030-12-29</t>
+        </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Medium haul: range check, services per day; E175 and E190 in the shop</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>Week 3</t>
-        </is>
-      </c>
+          <t>Chapter 1 review: chapter accounts by hand; the long-haul decision</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr"/>
       <c r="D11" s="13" t="inlineStr">
         <is>
           <t>live</t>
@@ -22165,85 +22572,71 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="n">
-        <v>22</v>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Week-at-a-time play; load factor %; event costs as a share of profit; weekly review</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>Week 4</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2031-01-06</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>CHAPTER 2: long haul, overnight rotations, time zones; leasing; reputation revealed; airline type; Value extras; crew cost by type; Captain's challenges; hunts</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>placeholder</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2030-12-02</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Month-at-a-time play; monthly reports from here on</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>Chapter 1 run</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>2031-08-31</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Chapter 2 review</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>placeholder</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>2030-12-28</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Chapter 1 review: chapter accounts by hand; the long-haul decision</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>2031-09-02</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>CHAPTER 3: buy outright; overdraft safety net</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>placeholder</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>2031-01-06</t>
+          <t>2032-08-31</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>CHAPTER 2 set-up: long haul, overnight rotations, time zones; leasing (standing); reputation revealed; airline type; Value extras; Captain's challenges begin</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>Chapter 2</t>
-        </is>
-      </c>
+          <t>Chapter 3 review</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr"/>
       <c r="D15" s="14" t="inlineStr">
         <is>
           <t>placeholder</t>
@@ -22251,87 +22644,71 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>2031-08-31</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>Chapter 2 review: year-1 accounts, first hunt, next investment</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>placeholder</t>
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>2032-09-07</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>CHAPTER 4: A380 on finance; reputation that matters</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr"/>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>later</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>2031-09-02</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>CHAPTER 3 set-up: buy outright (price − cash, ÷ profit a week); overdraft safety net</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>Chapter 3</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>placeholder</t>
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>2033-08-31</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Chapter 4 review</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr"/>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>later</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>2032-08-31</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Chapter 3 review</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>placeholder</t>
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>2033-09-06</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>CHAPTER 5: rival enters the best route; marketing; quarterly comparison task</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr"/>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>later</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t>2032-09-07</t>
+          <t>2034-08-31</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>CHAPTER 4 set-up: the A380; reputation that moves demand; finance (deposit, weekly repayments)</t>
-        </is>
-      </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>Chapter 4</t>
-        </is>
-      </c>
+          <t>Chapter 5 review</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr"/>
       <c r="D19" s="18" t="inlineStr">
         <is>
           <t>later</t>
@@ -22341,19 +22718,15 @@
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
         <is>
-          <t>2033-08-31</t>
+          <t>2034-09-05</t>
         </is>
       </c>
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>Chapter 4 review</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
+          <t>CHAPTER 6: no new mechanic; the five-year review</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr"/>
       <c r="D20" s="18" t="inlineStr">
         <is>
           <t>later</t>
@@ -22361,128 +22734,22 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>2033-09-06</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>CHAPTER 5 set-up: rival enters the best route; marketing; quarterly comparison task</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>Chapter 5</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>later</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>2034-08-31</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Chapter 5 review</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>later</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>2034-09-05</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>CHAPTER 6: no new mechanic; the five-year review builds through the year</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>Chapter 6</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>later</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>2035-08-31</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Five-year review: graphs and averages</t>
-        </is>
-      </c>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>End</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>later</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>rule</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>Reports follow the time step (D40); hand sums follow HandSumRules (D34); cash rules D26 with no overdraft charge (F7)</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr"/>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>rule</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>No second hub, no sell-back, no fleet renewal, no investor; Heathrow only; Luton via the April 2031 event</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>D25 D31 D32 D44 D46</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>No crew mechanic before 2031-01-06; no second hub, sell-back, fleet renewal, investor; Heathrow only; cash reserve block before Sep 2031; HandSumRules govern hand sums</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>D51 D31 D25 D46 D44 D32 D26 D34</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>live</t>
         </is>
@@ -24149,11 +24416,11 @@
         </is>
       </c>
       <c r="E2" s="13" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="F2" s="13" t="inlineStr">
         <is>
-          <t>day → week (from day 22) → month (from Dec)</t>
+          <t>week (plan → run → review) to day 28; week-skips from day 29; months from 2030-12-02</t>
         </is>
       </c>
       <c r="G2" s="13" t="inlineStr">
@@ -24163,12 +24430,12 @@
       </c>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Running an airline: fare, services, timetable, fuel, time of day, two routes, a second plane, medium haul</t>
+          <t>Running an airline a week at a time: the standing plan on one page (timetable with demand curve, fare, snacks, fuel), the week on the operations board, the weekly review</t>
         </is>
       </c>
       <c r="I2" s="13" t="inlineStr">
         <is>
-          <t>timetable; snacks; fuel; rival fares; crew duty; weekends; second plane (buy or lease, tutorial tier); seasons; medium haul; £5 fares; load factor % (day 22); scaled event costs (day 22)</t>
+          <t>Launch Day: timetable, fare, snacks, fuel, both routes, modelling tool, workings page; week 2: second plane, rent-or-buy, launch-deal finance; week 3: four routes, £5 fares, seasons, use-it-or-lose-it; week 4: medium haul, range, E175/E190, load factor %; from week 5: weekly skips, Marrakech, the autumn pairs, scaled event costs</t>
         </is>
       </c>
       <c r="J2" s="13" t="n">
@@ -24784,7 +25051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -25294,11 +25561,11 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>From day 22 (week 4) an event's cost is costShare × yesterday's profit, rounded to £10 and printed on the card (D21). Days 1–21 use the fixed cash column.</t>
+          <t>D21: fixed pounds through week 4 (the four fully written events); costShare from week 5 (day 29).</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
@@ -25318,7 +25585,7 @@
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Load factor shown as a percentage from the first weekly review; before that '15 of 19' and empty seats only (D23).</t>
+          <t>D23: from the week-4 review.</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
@@ -25620,7 +25887,7 @@
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>HandSumRules rule 2: fuel is asked by hand when the price has moved 50p or more since it was last asked.</t>
+          <t>HandSumRules rule 2. Launch Day's fuel sum is done at Wednesday's price (£1.30); the next by hand is the week of 14 October (£3.00).</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
@@ -25904,84 +26171,260 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="23" t="inlineStr">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>openingPlayMode</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>week</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>D52: in chapter 1 the pupil builds a standing plan on one page, the week runs day by day on the operations board pausing only for events, and ends with a seven-row table, the total by hand and projected against actual. Day-by-day play remains a teacher option (teacherDayByDay).</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>teacherDayByDay</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>Teacher panel: TRUE runs chapter 1 a day at a time instead of a week at a time.</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>weeklyReviewFromDay</t>
+        </is>
+      </c>
+      <c r="B56" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>Every week ends with a review: seven-row table, total by hand, projected − actual, missed-profit line.</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>missedProfitLine</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>D55: the weekly review shows 'your plan £X · best plan available with your planes £Y · missed £Z', from the engine's plan sweep. No cash is taken.</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>neglectFromDay</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>D55 use-it-or-lose-it: from week 3, a route with no service for a week, or flown under neglectLoadFactor all week, loses neglectLossShare of its passengers to Red Kite the next week; it recovers neglectRecoverShare a week once flown properly. The review names the route.</t>
+        </is>
+      </c>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>neglectLoadFactor</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C59" s="13" t="inlineStr"/>
+      <c r="D59" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>neglectLossShare</t>
+        </is>
+      </c>
+      <c r="B60" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>A tenth: the sum stays in tenths.</t>
+        </is>
+      </c>
+      <c r="D60" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>neglectRecoverShare</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C61" s="13" t="inlineStr"/>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>launchDaySums</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>tickets ×3 fares; profit; snacks ×2 prices; fuel after a guided example</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>D54: all on Launch Day, in one sitting, on the workings page, in this order.</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>practiceQuestionsPerDay</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>Teacher panel: 0 | 1 | 3. Practice questions use the pupil's own numbers and appear after the plan sums, marked optional (Design Note 8 Oct).</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="23" t="inlineStr">
         <is>
           <t>blockedFlightCodes</t>
         </is>
       </c>
-      <c r="B54" s="23" t="inlineStr">
+      <c r="B64" s="23" t="inlineStr">
         <is>
           <t>BA, EZ, FR, VS, LH, AF, KL, U2</t>
         </is>
       </c>
-      <c r="C54" s="23" t="inlineStr">
+      <c r="C64" s="23" t="inlineStr">
         <is>
           <t>CR5. Real airline codes the pupil cannot pick; refused calmly ("That code belongs to a real airline, try another").</t>
         </is>
       </c>
-      <c r="D54" s="23" t="inlineStr">
+      <c r="D64" s="23" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="23" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="23" t="inlineStr">
         <is>
           <t>soundDefault</t>
         </is>
       </c>
-      <c r="B55" s="23" t="inlineStr">
+      <c r="B65" s="23" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="C55" s="23" t="inlineStr">
+      <c r="C65" s="23" t="inlineStr">
         <is>
           <t>CR5. Sound (take-off, airport chimes, announcements) is off until the teacher turns it on; a mute control sits in the top bar.</t>
         </is>
       </c>
-      <c r="D55" s="23" t="inlineStr">
+      <c r="D65" s="23" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="23" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="23" t="inlineStr">
         <is>
           <t>revealSeconds</t>
         </is>
       </c>
-      <c r="B56" s="23" t="n">
+      <c r="B66" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="C56" s="23" t="inlineStr">
+      <c r="C66" s="23" t="inlineStr">
         <is>
           <t>CR5. The hangar reveal on launch day: doors close, open, the plane rolls in. Later planes get about half.</t>
         </is>
       </c>
-      <c r="D56" s="23" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="23" t="inlineStr">
-        <is>
-          <t>practiceQuestionsPerDay</t>
-        </is>
-      </c>
-      <c r="B57" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="C57" s="23" t="inlineStr">
-        <is>
-          <t>Design note 8 Oct. Optional practice questions after the day's sums on the workings page, with the pupil's own numbers: 0, 1 or 3 (the teacher panel can change it).</t>
-        </is>
-      </c>
-      <c r="D57" s="23" t="inlineStr">
+      <c r="D66" s="23" t="inlineStr">
         <is>
           <t>live</t>
         </is>
@@ -26844,7 +27287,7 @@
         <v>0.2</v>
       </c>
       <c r="P4" s="12" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="Q4" s="12" t="inlineStr">
         <is>
@@ -26918,7 +27361,7 @@
         <v>0.15</v>
       </c>
       <c r="P5" s="12" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="12" t="inlineStr">
         <is>
@@ -26992,7 +27435,7 @@
         <v>0.15</v>
       </c>
       <c r="P6" s="12" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="Q6" s="12" t="inlineStr">
         <is>
@@ -27066,7 +27509,7 @@
         <v>0.25</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="Q7" s="12" t="inlineStr">
         <is>
@@ -27140,7 +27583,7 @@
         <v>0.2</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="Q8" s="12" t="inlineStr">
         <is>
@@ -27214,7 +27657,7 @@
         <v>0.2</v>
       </c>
       <c r="P9" s="12" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="Q9" s="12" t="inlineStr">
         <is>
@@ -27436,7 +27879,7 @@
         <v>0.2</v>
       </c>
       <c r="P12" s="13" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
@@ -27510,7 +27953,7 @@
         <v>0.2</v>
       </c>
       <c r="P13" s="13" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
@@ -27584,7 +28027,7 @@
         <v>0.2</v>
       </c>
       <c r="P14" s="13" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
@@ -27658,7 +28101,7 @@
         <v>0.25</v>
       </c>
       <c r="P15" s="13" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
@@ -27732,7 +28175,7 @@
         <v>0.25</v>
       </c>
       <c r="P16" s="13" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
@@ -27806,7 +28249,7 @@
         <v>0.25</v>
       </c>
       <c r="P17" s="13" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
@@ -27880,7 +28323,7 @@
         <v>0.2</v>
       </c>
       <c r="P18" s="13" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
@@ -27954,7 +28397,7 @@
         <v>0.2</v>
       </c>
       <c r="P19" s="13" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
@@ -28028,7 +28471,7 @@
         <v>0.15</v>
       </c>
       <c r="P20" s="13" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
@@ -28102,7 +28545,7 @@
         <v>0.2</v>
       </c>
       <c r="P21" s="13" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
@@ -28248,7 +28691,7 @@
         </is>
       </c>
       <c r="J2" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K2" s="15" t="inlineStr">
         <is>
@@ -28304,7 +28747,7 @@
         </is>
       </c>
       <c r="J3" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K3" s="15" t="inlineStr">
         <is>
@@ -28360,7 +28803,7 @@
         </is>
       </c>
       <c r="J4" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K4" s="15" t="inlineStr">
         <is>
@@ -28416,7 +28859,7 @@
         </is>
       </c>
       <c r="J5" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K5" s="15" t="inlineStr">
         <is>
@@ -28472,7 +28915,7 @@
         </is>
       </c>
       <c r="J6" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
@@ -28528,7 +28971,7 @@
         </is>
       </c>
       <c r="J7" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K7" s="15" t="inlineStr">
         <is>
@@ -28584,7 +29027,7 @@
         </is>
       </c>
       <c r="J8" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K8" s="15" t="inlineStr">
         <is>
@@ -28640,7 +29083,7 @@
         </is>
       </c>
       <c r="J9" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
@@ -28696,7 +29139,7 @@
         </is>
       </c>
       <c r="J10" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10" s="15" t="inlineStr">
         <is>
@@ -28752,7 +29195,7 @@
         </is>
       </c>
       <c r="J11" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
@@ -28808,7 +29251,7 @@
         </is>
       </c>
       <c r="J12" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K12" s="15" t="inlineStr">
         <is>
@@ -28864,7 +29307,7 @@
         </is>
       </c>
       <c r="J13" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
@@ -29544,10 +29987,10 @@
         <v>150</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="J2" s="12" t="n">
-        <v>5000</v>
+        <v>12000</v>
       </c>
       <c r="K2" s="12" t="n">
         <v>2500</v>
@@ -29607,10 +30050,10 @@
         <v>200</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>9000</v>
+        <v>22000</v>
       </c>
       <c r="K3" s="12" t="inlineStr"/>
       <c r="L3" s="12" t="n">
@@ -29668,10 +30111,10 @@
         <v>350</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>1200</v>
+        <v>1800</v>
       </c>
       <c r="J4" s="12" t="n">
-        <v>15000</v>
+        <v>36000</v>
       </c>
       <c r="K4" s="12" t="inlineStr"/>
       <c r="L4" s="12" t="n">
@@ -29729,14 +30172,14 @@
         <v>900</v>
       </c>
       <c r="I5" s="12" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="J5" s="12" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="K5" s="12" t="inlineStr"/>
       <c r="L5" s="12" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="M5" s="12" t="inlineStr">
         <is>
@@ -29797,7 +30240,7 @@
       </c>
       <c r="K6" s="12" t="inlineStr"/>
       <c r="L6" s="12" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="M6" s="12" t="inlineStr">
         <is>
@@ -29858,7 +30301,7 @@
       </c>
       <c r="K7" s="12" t="inlineStr"/>
       <c r="L7" s="12" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
@@ -29919,7 +30362,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr"/>
       <c r="L8" s="12" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="M8" s="12" t="inlineStr">
         <is>
@@ -30259,14 +30702,14 @@
         <v>700</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="K15" s="13" t="n"/>
       <c r="L15" s="13" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="M15" s="13" t="inlineStr">
         <is>
@@ -30485,7 +30928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30571,24 +31014,22 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>5000</v>
+        <v>12000</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>250</v>
       </c>
       <c r="D2" s="13" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="E2" s="13" t="n">
         <v>300</v>
       </c>
       <c r="F2" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>launch deal</t>
-        </is>
+        <v>30</v>
+      </c>
+      <c r="G2" s="13" t="n">
+        <v>13000</v>
       </c>
       <c r="H2" s="13" t="inlineStr">
         <is>
@@ -30597,7 +31038,7 @@
       </c>
       <c r="I2" s="13" t="inlineStr">
         <is>
-          <t>day 1</t>
+          <t>day 8</t>
         </is>
       </c>
       <c r="J2" s="13" t="inlineStr">
@@ -30607,7 +31048,7 @@
       </c>
       <c r="K2" s="13" t="inlineStr">
         <is>
-          <t>Second Twin Otter: rent £250 a day or buy £5,000 → 20 days. Launch-deal finance kept: £2,000 down, £300 a day for 12 days (days, not weeks).</t>
+          <t>Second Twin Otter: rent £250 a day; 12,000 ÷ 250 = 48 days. Launch-deal finance £4,000 down, £300 a day for 30 days (£13,000).</t>
         </is>
       </c>
       <c r="L2" s="13" t="inlineStr">
@@ -30623,24 +31064,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>9000</v>
+        <v>22000</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>400</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>3000</v>
+        <v>7000</v>
       </c>
       <c r="E3" s="13" t="n">
         <v>500</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>launch deal</t>
-        </is>
+        <v>32</v>
+      </c>
+      <c r="G3" s="13" t="n">
+        <v>23000</v>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
@@ -30659,7 +31098,7 @@
       </c>
       <c r="K3" s="13" t="inlineStr">
         <is>
-          <t>The week-2 lesson: 9,000 ÷ 400 = 22½ days. Launch-deal finance £3,000 down, £500 a day for 14 days.</t>
+          <t>The week-2 sum: 22,000 ÷ 400 = 55 days. Launch-deal finance £7,000 down, £500 a day for 32 days (£23,000). Buy greyed out until cash ≥ price + reserve.</t>
         </is>
       </c>
       <c r="L3" s="13" t="inlineStr">
@@ -30675,24 +31114,22 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>15000</v>
+        <v>36000</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>650</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>5000</v>
+        <v>11000</v>
       </c>
       <c r="E4" s="13" t="n">
         <v>800</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>launch deal</t>
-        </is>
+        <v>35</v>
+      </c>
+      <c r="G4" s="13" t="n">
+        <v>39000</v>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
@@ -30711,7 +31148,7 @@
       </c>
       <c r="K4" s="13" t="inlineStr">
         <is>
-          <t>Launch-deal finance £5,000 down, £800 a day for 14 days.</t>
+          <t>36,000 ÷ 650 ≈ 55 days. Finance £11,000 down, £800 a day for 35 days (£39,000).</t>
         </is>
       </c>
       <c r="L4" s="13" t="inlineStr">
@@ -30727,33 +31164,31 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>900</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>7000</v>
+        <v>15000</v>
       </c>
       <c r="E5" s="13" t="n">
         <v>1000</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>launch deal</t>
-        </is>
+        <v>38</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>53000</v>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>day 15</t>
+          <t>day 22</t>
         </is>
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>day 15</t>
+          <t>day 22</t>
         </is>
       </c>
       <c r="J5" s="13" t="inlineStr">
@@ -30763,7 +31198,7 @@
       </c>
       <c r="K5" s="13" t="inlineStr">
         <is>
-          <t>Tutorial jet. 20,000 ÷ 900 ≈ 22 days.</t>
+          <t>50,000 ÷ 900 ≈ 56 days. Finance £15,000 down, £1,000 a day for 38 days (£53,000).</t>
         </is>
       </c>
       <c r="L5" s="13" t="inlineStr">
@@ -30779,33 +31214,31 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1200</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>10000</v>
+        <v>21000</v>
       </c>
       <c r="E6" s="13" t="n">
         <v>1500</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>launch deal</t>
-        </is>
+        <v>36</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>75000</v>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>day 15</t>
+          <t>day 22</t>
         </is>
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>day 15</t>
+          <t>day 22</t>
         </is>
       </c>
       <c r="J6" s="13" t="inlineStr">
@@ -30815,7 +31248,7 @@
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>Tutorial jet. 30,000 ÷ 1,200 = 25 days.</t>
+          <t>70,000 ÷ 1,200 ≈ 58 days. Finance £21,000 down, £1,500 a day for 36 days (£75,000).</t>
         </is>
       </c>
       <c r="L6" s="13" t="inlineStr">
@@ -31304,6 +31737,13 @@
       <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Note on the launch-deal rows: tutorial finance is in daily payments (as in the game today), because the opening is played by the day; from the A220 the payments are weekly, because chapter 4 is played by the month. 'When does renting cost more than buying?' = price ÷ leaseDaily: about 20–25 days for tutorial planes (launch deals), 1,000 days for every jet from the A220 up (F4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Tutorial prices are 2½× v4.3 (D55): the second plane is rented or financed in week 2 and bought outright around week 4–5. The first Twin Otter is still the £2,500 launch deal. Rent-or-buy ≈ 55 days for every tutorial plane; 1,000 days for jets from the A220 up.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook v4.9: cap, decay and floor settings (D63–D64)
Installs Fable's v4.9 (it carries the CR5 parts, so no merge is needed) and
adds the v4.7 and v4.9 settings to the importer's chapter-1 checks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013x87PezhtynWHJHngTWCer
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chapters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="HandSumRules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="WorkingMethods" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Settings" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="RouteNews" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Archetypes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Routes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="RouteCatalogue" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Aircraft" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Finance" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Airports" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Calendar" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Market" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Events" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Challenges" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Mechanics" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Catering" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Hunts" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Livery" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HandSumRules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkingMethods" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RouteNews" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archetypes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RouteCatalogue" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aircraft" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Airports" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Challenges" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catering" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hunts" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livery" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -719,6 +719,13 @@
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>v4.7 (12 Oct): D61 review totals and means are Build steps (show what to add, show the divisor); D62 second-aircraft comparison (Settings secondAircraftCompare, whereCouldItFly). Brief: Second aircraft and reviews.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>v4.9 (13 Oct): base is Claude Code's installed v4.7 (with the CR5 Livery sheet, Aircraft artworkId/photo columns and blockedFlightCodes/soundDefault/revealSeconds), so no merge script is needed from here. Adds D63 cap of three Calculate sign-offs a week from week 2 with repetition decay (HandSumRules 9–10, Settings signOffCapPerWeek, signOffDecayAfter) and D64 the floor: a monthly audit, becoming a board review with three sign-offs and a required change when the plan has not changed all month (HandSumRules 11, Settings auditFloor, boardNudge*). Brief: Cap, decay and floor.</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1517,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
@@ -1724,7 +1730,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
@@ -26895,7 +26900,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -26914,7 +26918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -27197,8 +27201,99 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>A cap of three a week from week 2</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>At most signOffCapPerWeek Calculate sign-offs in a week; the most instructive first; the rest Build or Model; overflow carried to the next relevant week. Launch Day and review Build steps are outside the cap.</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>weekly, from day 8</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>week 3: 34 × £95, 675 ÷ 450 and the Saab's Amsterdam fuel; Frankfurt, Geneva and Barcelona tickets as Build</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Sums get lighter with repetition</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Calculate the first two times a relationship appears; Build for a new instance from the third time; Model when nothing is new.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>relationship.count</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>tickets on a new route in week 4 is a Build (pick passengers, ×, fare), not a long multiplication</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>The floor: a monthly audit, and the board when nothing has changed</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>The world's penalties run all the time (missed profit, neglect, day costs, fuel, news). At each month end Finance sends one audit on the pupil's weakest line. If the plan has not changed all month, the audit becomes a board review: three sign-offs and a required change of plan before the next month runs.</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>month end; plan unchanged for 4 weeks</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>end of October: 'Finance: check the Geneva line before the accounts close'; a coasting pupil in November: 'The board wants to see a plan that tests a different fare or route'</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Rough count: chapter 1 about 25 hand sums, chapter 2 about 8, chapter 3 about 6, chapter 4 about 6, chapter 5 about 5, chapter 6 about 4 — roughly 55 over the game, half of them × or ÷, excluding challenges and hunts. The teacher's Calculate / Build / Model setting overrides any rule (D34).</t>
         </is>
@@ -27604,7 +27699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -29394,6 +29489,124 @@
         </is>
       </c>
       <c r="D86" s="23" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>signOffCapPerWeek</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>D63: from week 2, at most this many Calculate sign-offs in a week (teacher dial 1–3). Launch Day's sums and the review's Build steps are outside the cap. When more qualify, the game asks the most instructive first: a relationship never met, then a known relationship with a changed input (a fuel price jump), then the one with the most money in it; the rest are filled by the model with ƒ. A sum that misses the cap is carried to the next week it is relevant.</t>
+        </is>
+      </c>
+      <c r="D87" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>signOffDecayAfter</t>
+        </is>
+      </c>
+      <c r="B88" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" s="13" t="inlineStr">
+        <is>
+          <t>D63: a relationship is Calculate the first two times it appears; a new instance from the third time (tickets on a new route, fuel for a new plane) is Build; once nothing is new it is Model. The teacher can hold any relationship at Calculate.</t>
+        </is>
+      </c>
+      <c r="D88" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>auditFloor</t>
+        </is>
+      </c>
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>D64: at each month end Finance sends an audit — re-check one existing figure from the pupil's own airline, chosen as the route with the most missed profit. Falls on the last day of each month; from December it comes with the monthly report.</t>
+        </is>
+      </c>
+      <c r="D89" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>boardNudgeIdleWeeks</t>
+        </is>
+      </c>
+      <c r="B90" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C90" s="13" t="inlineStr">
+        <is>
+          <t>D64: if the standing plan has not changed for a month, the month-end audit becomes a board review: three sign-offs (re-check two lines and the month's average day) and the board asks for a plan that tests a different fare or route before the next month runs.</t>
+        </is>
+      </c>
+      <c r="D90" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>boardNudgeMissedShare</t>
+        </is>
+      </c>
+      <c r="B91" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C91" s="13" t="inlineStr">
+        <is>
+          <t>Missed profit as a share of the best plan available, over the month.</t>
+        </is>
+      </c>
+      <c r="D91" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>boardReviewSignOffs</t>
+        </is>
+      </c>
+      <c r="B92" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C92" s="13" t="inlineStr"/>
+      <c r="D92" s="13" t="inlineStr">
         <is>
           <t>live</t>
         </is>

</xml_diff>

<commit_message>
Workbook v4.11 and D67: a Days setting on every flight (revised Studio)
- Workbook v4.11 installed; importer checks the six new settings.
- p4zf_flightdays.js (v2 build only): each flight is All week, Mon-Fri or
  Sat-Sun from day 8. The engine prices each day with its own flights;
  departures and the duty day are checked per day type; plans, keys,
  moves, deletes and adds carry the days.
- Revised Studio: Mon-Fri | Sat-Sun timetable switch, chips on blocks,
  Days in the flight and route editors, split seat fill in the summary,
  opener and Sunday review, weekend-only news presets a Sat-Sun service,
  PlanTips weekend_only_news and fare_lower_fills.
- week.test.js: the rugby-week Sat-Sun Dublin check (v2 mode).
- Docs: README, State of the Game, Flight-Days-Report-Back.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013x87PezhtynWHJHngTWCer
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -734,6 +734,13 @@
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>v4.10 (13 Oct): D66 Operating Plan Studio data — seat-fill thresholds (Settings seatFillGood/Medium), per-route demand strip (demandStripMode), the four-step bar (planStudioSteps), and the PlanTips sheet (ten data-driven live tips). Data appendix: Operating Plan Studio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>v4.11 (13 Oct): D67 flight Days setting (All week / Mon–Fri / Sat–Sun) from week 2, weekday and weekend seat fill shown separately, patterns may be a day plus extras; haul-band settings; PlanTips gains fare_lower_fills and weekend_only_news.</t>
         </is>
       </c>
     </row>
@@ -28972,7 +28979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -30960,6 +30967,124 @@
         </is>
       </c>
       <c r="D96" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>flightDays</t>
+        </is>
+      </c>
+      <c r="B97" s="13" t="inlineStr">
+        <is>
+          <t>All week | Mon–Fri | Sat–Sun</t>
+        </is>
+      </c>
+      <c r="C97" s="13" t="inlineStr">
+        <is>
+          <t>D67: every flight in a standing plan has a Days setting, default All week, set in the flight editor. Weekend-only services exist for news such as the Dublin rugby; weekday-only services suit business routes that are quiet on Saturdays.</t>
+        </is>
+      </c>
+      <c r="D97" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>flightDaysFromDay</t>
+        </is>
+      </c>
+      <c r="B98" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="C98" s="13" t="inlineStr">
+        <is>
+          <t>The Days setting appears from week 2 (Launch Day keeps one timetable for the week).</t>
+        </is>
+      </c>
+      <c r="D98" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>summaryWeekdayWeekend</t>
+        </is>
+      </c>
+      <c r="B99" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C99" s="13" t="inlineStr">
+        <is>
+          <t>D67: the summary bar and the Sunday review show seat fill for weekdays and the weekend separately when any flight is not All week.</t>
+        </is>
+      </c>
+      <c r="D99" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>patternPlusExtras</t>
+        </is>
+      </c>
+      <c r="B100" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C100" s="13" t="inlineStr">
+        <is>
+          <t>D67: a regular operating pattern is a whole day, and an aircraft may fly a pattern plus extra flights (for example Pattern A all week plus a Saturday Dublin service).</t>
+        </is>
+      </c>
+      <c r="D100" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>shortHaulMaxKm</t>
+        </is>
+      </c>
+      <c r="B101" s="13" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C101" s="13" t="inlineStr">
+        <is>
+          <t>Haul bands for the network filters (from Claude Code's revised Studio): short haul up to 1,500 km, medium to 4,000 km, long beyond.</t>
+        </is>
+      </c>
+      <c r="D101" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>mediumHaulMaxKm</t>
+        </is>
+      </c>
+      <c r="B102" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C102" s="13" t="inlineStr"/>
+      <c r="D102" s="13" t="inlineStr">
         <is>
           <t>live</t>
         </is>
@@ -30976,7 +31101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -31319,8 +31444,69 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>fare_lower_fills</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Seats are empty on a route and more people want to fly at the next fare down</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>{route} could fill all {seats} seats at £{lower}, but would earn £{diff} less per passenger.</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>weekend_only_news</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Announced news lifts a route's demand on the weekend only and the plan has no Sat–Sun service on it</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>{route} is busy this weekend only: add a Sat–Sun service rather than one all week.</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>D66: the Live seat fill panel shows at most two tips, lowest priority number first. Conditions are evaluated on the projected plan every time it changes; the same conditions feed the Sunday review's explanation of missed profit.</t>
         </is>

</xml_diff>

<commit_message>
Smoother first take-off; Workbook v5.1 (Bettws statement codes)
- The launch-day take-off is one continuous motion: taxi in and ease
  to a stop, line up, accelerate down the runway, rotate and climb out.
  Transforms only, drawn each frame from the start time, so a redrawn
  screen or the whiteboard picks up where it was. The old keyframes
  eased between each stage, which made the plane stop and start.
- Install Workbook v5.1. The importer reads
  WorkingMethods.bettwsStatements (the codes, and the text) and ignores
  the 'live' left in the notes of the six new rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013x87PezhtynWHJHngTWCer
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -748,6 +748,13 @@
       <c r="A25" s="10" t="inlineStr">
         <is>
           <t>v5.0 (13 Oct): CHAPTER 2 LIVE. New York and Dubai (unlockDay 127), Toronto (183), Lagos (218), Delhi (274, the first overnight rotation); a long_haul archetype (one flight a day, one in ten time-locked, growth 5% a week to ×1.5); the 757 and 787 live to lease, the 787 re-costed to be cheaper per seat than the 757 (130 L/100 km, £2,000/h, £6,000/day); A320/737 range 5,500 km and A220 5,000 so the Atlantic needs a long-haul plane; same-day long haul to 6,000 km with a £500 second crew; reputation ×5% a half-star from January with the autumn's stars banked; light airline types (Premium two higher fares and faster stars, Value one lower fare and the £20 bag fee at four in ten); demand tables extended a step below and two above every live route's options; fuel forecasts weeks 18–52; 19 route-news items January–August; the spring and summer events written with options; Challenges 1–2 and Hunts h1–h2 live; chapter-2 Calendar days 127–133. Balance Report v5.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>v5.1 (13 Oct): D75 pupil record — WorkingMethods gains bettwsStatements (WPS 3 + PFA codes per kind of sum) and six more rows (time, flight time, local time, reading reports, multipliers, the aircraft comparison) so every printed entry can carry its statements. Brief: Pupil record and printout.</t>
         </is>
       </c>
     </row>
@@ -28170,7 +28177,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
@@ -29549,7 +29555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -29558,6 +29564,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -29591,6 +29598,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>bettwsStatements (WPS 3 + PFA)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -29623,6 +29635,11 @@
           <t>Short × then × 10 for £10 fares; long × for £5 fares and fares over £100</t>
         </is>
       </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>NCP-3-06 · NCP-3-04 · ALG-3-08 (partition) · MON-3-02</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -29655,6 +29672,11 @@
           <t>Scale from 100 L: 100 L costs £147, so 20 L costs £29.40</t>
         </is>
       </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>NCP-3-06 · NCP-3-05 (decimals) · ALG-3-08 (partition the price) · FDP-3-06 (estimate first, check it looks right)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -29683,6 +29705,11 @@
         </is>
       </c>
       <c r="F4" s="13" t="inlineStr"/>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>NCP-3-05 · MON-3-02 · MON-3-01 · PFA-MM-02</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -29715,6 +29742,11 @@
           <t>D61: Build, not Calculate</t>
         </is>
       </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>NCP-3-05 · STAT-3-19 (totals and differences from data) · STAT-3-23 (the mean) · MON-3-01 · PFA-MM-02</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -29747,6 +29779,11 @@
           <t>Shown in the 'What changed?' panel</t>
         </is>
       </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>NCP-3-05 · STAT-3-19 · STAT-3-18 (reading the comparison) · MON-3-02</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -29775,6 +29812,11 @@
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>NCP-3-06 · NCP-3-02 (large numbers) · MON-3-01 · PFA-MM-02</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -29807,6 +29849,11 @@
           <t>'Saved compared with buying later', never profit</t>
         </is>
       </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>STAT-3-18 (reading a table) · STAT-3-25 (what the data cannot tell us) · MON-3-03 · PFA-MM-07 · FDP-3-06</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -29835,6 +29882,11 @@
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr"/>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>NCP-3-06 (division, remainders) · MON-3-03 (best value, price per unit) · PFA-MM-07</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -29863,6 +29915,11 @@
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>FDP-3-02 · FDP-3-03 (fraction as division) · FDP-3-01 (everyday set) · FDP-3-04</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -29891,6 +29948,11 @@
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr"/>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>FDP-3-02 · FDP-3-01 (one tenth = 10%) · FDP-3-03</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -29919,11 +29981,246 @@
           <t>Monthly reports from December; quarterly task later</t>
         </is>
       </c>
-    </row>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>STAT-3-23 (the mean) · STAT-3-19 · STAT-3-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>time: service length, departures, duty day</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Planning board; performance card</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>adding mixed hours and minutes; counting on</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>1 h + 45 min + 1 h + 35 min = 3 h 20; 06:30 to 21:15</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>TTT-3-01 · TTT-3-04 · CN-3-01 (reading a timetable) · DUR-3-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>flight time: distance ÷ speed</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Performance card; route card</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>short division; reasoning from multiplication facts</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>1,350 ÷ 450 = 3 h</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>NCP-3-06 · NCP-3-04 · DUR-3-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>local time: departure + flight + time zone</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Arrival card (long haul)</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>number line across the day</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>06:30 + 6 h 15 − 5 h = 07:45 New York time</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>TTT-3-01 · TTT-3-02 · NCP-3-03 (through zero / negative offsets)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>reading the World report and the review</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Monday plan page; Sunday review</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>reading graphs and tables; comparing projected with actual</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>fuel line, demand bars, seat-fill bars</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>STAT-3-18 · STAT-3-19 · STAT-3-24 · STAT-3-25 · PROB-3-03 (expected against what happened)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>reputation and news multipliers</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Review; route cards</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>percentage of an amount</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>4½ stars: 3 × 5% = 15% more; Paris ×0.4 in strike week</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>FDP-3-02 · PFA-MM-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>second-aircraft comparison</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>strategic</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Aircraft comparison (week 2)</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>reading a comparison table; seat-dot grids; cash bar; payback by division</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>22,000 − 13,000; 22,000 ÷ 590</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>STAT-3-18 · STAT-3-35 · MON-3-03 · MON-3-01 · NCP-3-06 · PFA-MM-04 (wants, needs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>D60: the workbench (Work it out) offers the methods listed for the relationship being signed off; the pupil chooses. Levels: operational (what does this one thing cost? — taught and calculated), model (what happens if I change this? — the console calculates), strategic (what should I do when the future is uncertain? — maths supports judgement).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Statement codes are from Bettws-Master-Dataset-v1_21 (WPS 3 main curriculum and PFA Managing Money). Drafted by Fable 13 Oct for Bertie to check; the pupil record prints these codes against each entry.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Install workbook v5.7 (D87 decision support, D88 what was it worth): importer reads the PlanTips action, moneyAtStake and experiment columns
The report lists the nine new Settings rows (operationsCheck, blockPreview, missedProfitDisplay, reviewFixLink,
planningSupport, experimentFlow, helpMeInvestigate, planImprovedBanner, whatWasItWorth) and the tips with their
priorities and experiments. 0 to fix, 21 to check. The game does not read them yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013x87PezhtynWHJHngTWCer
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -792,6 +792,13 @@
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>v5.6 (15 Oct): D86 working on paper — the workbench is an answer box, methods are reference cards; the two-tries rule; fuel is one sum a week (the Monday order, blocks × price per 1,000 L, by hand only on a 50p move) with the bill broken down by route and plane automatically; Launch Day keeps five sums (snacks as Build); cap of three a week confirmed. HandSumRules 2, 4 and 12. Every sum is numbered (Settings sumNumbering) so paper working matches the record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>v5.7 (15 Oct): D87 decision support — PlanTips gains action, moneyAtStake and experiment columns plus plane_unused, loss_making_service and plan_loses_money; Settings operationsCheck, blockPreview, missedProfitDisplay (words for the pupil, figures for the teacher), reviewFixLink, planningSupport dial (guided | supported | independent | management), experimentFlow, helpMeInvestigate, planImprovedBanner. Brief: Decision support. D88 'what was it worth?' (Settings whatWasItWorth; WorkingMethods row).</t>
         </is>
       </c>
     </row>
@@ -34716,7 +34723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -35152,6 +35159,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
@@ -35745,14 +35753,51 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr">
-        <is>
-          <t>D60: the workbench (Work it out) offers the methods listed for the relationship being signed off; the pupil chooses. Levels: operational (what does this one thing cost? — taught and calculated), model (what happens if I change this? — the console calculates), strategic (what should I do when the future is uncertain? — maths supports judgement).</t>
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>what a change was worth</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Plan improved banner; experiment compare; Sunday review</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>change per unit × units; then × 7 for the week</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>£20 × 57 = £1,140 a day; × 7 = £7,980 a week</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>NCP-3-06 · NCP-3-04 · MON-3-02 · PFA-MM-07</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>D60: the workbench (Work it out) offers the methods listed for the relationship being signed off; the pupil chooses. Levels: operational (what does this one thing cost? — taught and calculated), model (what happens if I change this? — the console calculates), strategic (what should I do when the future is uncertain? — maths supports judgement).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Statement codes are from Bettws-Master-Dataset-v1_21 (WPS 3 main curriculum and PFA Managing Money). Drafted by Fable 13 Oct for Bertie to check; the pupil record prints these codes against each entry.</t>
         </is>
@@ -35769,7 +35814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D139"/>
+  <dimension ref="A1:D148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -38643,6 +38688,194 @@
         </is>
       </c>
       <c r="D139" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="13" t="inlineStr">
+        <is>
+          <t>operationsCheck</t>
+        </is>
+      </c>
+      <c r="B140" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C140" s="13" t="inlineStr">
+        <is>
+          <t>D87: before Run week, a check shows the one or two PlanTips with the most money at stake, each with its action and 'Run anyway'. Never blocks; the action is the visually dominant button.</t>
+        </is>
+      </c>
+      <c r="D140" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="13" t="inlineStr">
+        <is>
+          <t>blockPreview</t>
+        </is>
+      </c>
+      <c r="B141" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C141" s="13" t="inlineStr">
+        <is>
+          <t>D87: a service block shows its expected fill while being moved (Earlier / Later or drag) and a one-line 'this change: seats a → b, profit £x → £y' after the drop; a full service with passengers turned away shows the fare chips with expected fill at each.</t>
+        </is>
+      </c>
+      <c r="D141" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="13" t="inlineStr">
+        <is>
+          <t>missedProfitDisplay</t>
+        </is>
+      </c>
+      <c r="B142" s="13" t="inlineStr">
+        <is>
+          <t>words for the pupil; figures for the teacher</t>
+        </is>
+      </c>
+      <c r="C142" s="13" t="inlineStr">
+        <is>
+          <t>D87: the pupil's review says 'a large improvement is available' (gap &gt; 30% of the best), 'a better plan is available' (10–30%) or 'a good plan' (&lt; 10%); the exact best-plan figure appears on the teacher panel and the printed review only.</t>
+        </is>
+      </c>
+      <c r="D142" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="13" t="inlineStr">
+        <is>
+          <t>reviewFixLink</t>
+        </is>
+      </c>
+      <c r="B143" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C143" s="13" t="inlineStr">
+        <is>
+          <t>D87: the Sunday review names the biggest missed opportunity (the tip with the most money at stake over the week) and offers 'Fix next week's {route} plan', which opens the carried-over plan with that route selected and its demand curve shown.</t>
+        </is>
+      </c>
+      <c r="D143" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="13" t="inlineStr">
+        <is>
+          <t>planningSupport</t>
+        </is>
+      </c>
+      <c r="B144" s="13" t="inlineStr">
+        <is>
+          <t>guided</t>
+        </is>
+      </c>
+      <c r="C144" s="13" t="inlineStr">
+        <is>
+          <t>D87: teacher dial — guided | supported | independent | management. guided: the check names the issue and offers 2–3 experiments (change the fare / the times / the number of services / the aircraft) with a prediction step; supported: names the issue only, the pupil chooses what to change; independent: shows the data and the modelling controls, no issue named; management: flags only losses and exceptions. Default guided for chapter 1; the dial is per pupil.</t>
+        </is>
+      </c>
+      <c r="D144" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="13" t="inlineStr">
+        <is>
+          <t>experimentFlow</t>
+        </is>
+      </c>
+      <c r="B145" s="13" t="inlineStr">
+        <is>
+          <t>choose variable → predict → change one thing → model → compare → decide</t>
+        </is>
+      </c>
+      <c r="C145" s="13" t="inlineStr">
+        <is>
+          <t>D87: in guided and supported levels every test is one variable at a time; the prediction (more / fewer / about the same seats; higher / lower / about the same profit) is recorded and compared; never a 'recommended' plan.</t>
+        </is>
+      </c>
+      <c r="D145" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="13" t="inlineStr">
+        <is>
+          <t>helpMeInvestigate</t>
+        </is>
+      </c>
+      <c r="B146" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C146" s="13" t="inlineStr">
+        <is>
+          <t>A small button on the plan and the review that reopens the guided experiment at any support level.</t>
+        </is>
+      </c>
+      <c r="D146" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="13" t="inlineStr">
+        <is>
+          <t>planImprovedBanner</t>
+        </is>
+      </c>
+      <c r="B147" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C147" s="13" t="inlineStr">
+        <is>
+          <t>D87: when the projected result improves after a change, a small 'Plan improved: seats a → b, result £x → £y' confirmation above Run week.</t>
+        </is>
+      </c>
+      <c r="D147" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="13" t="inlineStr">
+        <is>
+          <t>whatWasItWorth</t>
+        </is>
+      </c>
+      <c r="B148" s="13" t="inlineStr">
+        <is>
+          <t>change per unit × units = a day; × 7 = a week</t>
+        </is>
+      </c>
+      <c r="C148" s="13" t="inlineStr">
+        <is>
+          <t>D88: whenever the pupil changes a fare, a time or a service (in the plan or an experiment), show one line: fare — '£20 more a ticket × 57 passengers = £1,140 more a day'; time — '9 more passengers × £90 = £810 more a day'; service — 'one more flight: 19 × £90 − £615 costs = £1,095 a day'. The first time each kind appears it is a Build (tap the figures and ×), then Model; not counted in the sign-off cap. The Sunday review repeats it for the week ('Your Dublin fare rise was worth £7,980 this week'). Rule: the pupil sees figures for changes he made or tested; words for what is still available (missedProfitDisplay).</t>
+        </is>
+      </c>
+      <c r="D148" s="13" t="inlineStr">
         <is>
           <t>live</t>
         </is>
@@ -38659,7 +38892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -38668,6 +38901,9 @@
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -38701,6 +38937,21 @@
           <t>status</t>
         </is>
       </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>action (what the button opens)</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>moneyAtStake (rule)</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>experiment (guided)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -38731,6 +38982,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Show on timetable: highlight the band and the route's flights</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>profit of the best plan that adds one service in the band − current</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Change the times</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -38761,6 +39027,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Select this flight (Earlier / Later / Remove)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>profit with this flight at its best time − current</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Change the times</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -38791,6 +39072,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Test fare: show the fare chips with expected fill at each; or Add a service</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>max over fares and +1 service − current</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Change the fare | Change the number of services</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -38821,6 +39117,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Test fare: chips with expected fill</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>profit at the best fare − current</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Change the fare</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -38851,6 +39162,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Test next fare up</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>profit at the next fare − current</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Change the fare</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -38881,6 +39207,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Add a service in the idle time (opens + Service at that time)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>profit of the best added service</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Change the number of services</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -38911,6 +39252,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Open the route on the comparison (which plane suits it)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>profit with the best plane − current</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Change the aircraft</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -38941,6 +39297,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Open the aircraft comparison</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Change the aircraft</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -38971,6 +39342,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -39001,6 +39387,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -39031,6 +39432,21 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Test the lower fare</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>profit at the lower fare − current</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Change the fare</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -39061,11 +39477,168 @@
           <t>live</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Add a Sat–Sun service on the route</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>profit of the weekend service</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Change the number of services</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>plane_unused</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>A plane in the fleet has no flights in the standing plan</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>{plane} has no flights. It costs £{dayCost} a day parked.</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Find work for this aircraft (opens the timetable with the plane's row selected and + Service)</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>its day cost + profit of its best plan</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>Change the number of services | Change the aircraft</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>loss_making_service</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>A service's revenue is below its own flying, fuel, landing and passenger costs</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>{band} {route} loses £{loss} a trip.</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>Compare: remove / retime / reprice (three previews)</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>the loss, or the gain from the best of the three</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>Change the times | Change the fare | Change the number of services</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>plan_loses_money</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>The whole plan projects a loss for the day</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>This plan loses £{loss} a day. The biggest opportunity is {topTip}.</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Show me (opens the top tip's action)</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>the loss</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>D66: the Live seat fill panel shows at most two tips, lowest priority number first. Conditions are evaluated on the projected plan every time it changes; the same conditions feed the Sunday review's explanation of missed profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>D87: the Operations Check shows the one or two tips with the most money at stake (moneyAtStake rule, engine-computed), each with its action button; the pupil sees the words, never the best-plan figure. Priority 0–1 tips always rank first.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Screens brief 3 (D101, D102), work in progress: the teacher test toolkit, the one-flight demand rule and shape, flight times in hours and minutes, the fixed inspector and folded routes, results framing and the weekly graph, the worth check in the comparison, Coming up, the colour limit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013x87PezhtynWHJHngTWCer
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -14,26 +14,27 @@
     <sheet name="Settings" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="PlanTips" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="DailyColour" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Upgrades" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Briefings" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="RouteNews" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Archetypes" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="EventOptions" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Milestones" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Campaign" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Routes" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="RouteCatalogue" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Aircraft" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Finance" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Airports" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Calendar" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Market" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Events" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Challenges" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Mechanics" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Catering" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Hunts" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Livery" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Roadmap" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Upgrades" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Briefings" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="RouteNews" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Archetypes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="EventOptions" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Milestones" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Campaign" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Routes" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="RouteCatalogue" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Aircraft" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Finance" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Airports" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Calendar" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Market" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Events" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Challenges" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Mechanics" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Catering" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Hunts" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Livery" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -576,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -820,12 +821,660 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Took from v5.17 (17 Oct 2026, Claude Code): D101 and D102 only (Screens brief 3) — the Roadmap sheet; Settings adaptToOnlyFlight, demandShapeDisplay, flightTimeDecay, timeAnswerFormat, flightTimesTable, weekPlanTutorial, redMeans, opportunityDisplay, resultsFraming, flightInspector, activeRoutesCollapsible, weekGraphDefault, dailyColourLimit, comingUp, aircraftWorthCheck, teacherTestMode, and from D100 the three rows D101 builds on (waitCostLine, aircraftCardMeasure, demandStripMode); the fuel dips: Market weeks 3–5 and Calendar days 22–28. The rest of v5.16–v5.17 (D100, the D92 market from week 6 on) is kept in data/incoming/.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>briefingId</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>beat1 (show)</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>beat2 (predict: the pupil does…)</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>beat3 (reveal)</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>beat4 (use)</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>leadsInto</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="J1" s="20" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="K1" s="20" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>fare_lever</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Launch Day, the fare chips</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>What a fare does</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Nineteen passenger dots and a £ meter. The fare slides from £80 to £90 to £100; the meter per passenger rises as dots fade.</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>Drag the fare yourself; predict: more or fewer dots at £100?</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>Revenue = passengers × fare: both move. At £100 Paris wants 44, not 50 — two planes still fill.</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Back to the chips with the three revenue figures</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>Launch Day sum 1</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>briefing-fare.html</t>
+        </is>
+      </c>
+      <c r="K2" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>rival_split</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Thu, week 1 (Red Kite)</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Customers have a choice</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>62 Dublin dots; a red-kite plane lands beside yours; its price tag reads £50.</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Slide your fare; watch dots cross to Red Kite: 1 in 10 per £10.</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>The switching rule in one line; advertising halves it.</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>The Red Kite decision with the sum on it</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Red Kite card</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>briefing-rival.html</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>full_route</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Week-1 review</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>More demand than seats</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Passenger dots arrive at the terminal; 57 board three Twin Otters; the rest stay on the apron.</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Click the dots left behind; how many?</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>High demand is not profit if you cannot carry people: a bigger plane, another plane, or a higher fare.</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>The capacity observation and Compare aircraft</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>Week-2 decision</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>briefing-capacity.html</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>weekend_demand</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Week-2 review</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Weekdays and weekends</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Mon–Sun bars grow for Dublin; business icons fill weekdays, families the weekend.</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Click the days that look different.</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Why: business travel builds on weekdays; leisure swells at the weekend. Your timetable appears underneath — the same every day.</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Does the planner fit what the passengers do? → the Upgrades question</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>weekend_schedules upgrade</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>45</v>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>briefing-weekend.html</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>fuel_cash_tank_profit</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>First Fuel desk visit (day 8)</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Cash, tank, profit</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Three gauges: cash £12,409, tank 0 L, profit today. Press Buy 7,000 L: cash flows into the tank; profit does not move.</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Press Buy yourself; then: what changed? (tap the gauge)</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>A Twin Otter departs for Paris: 120 L drains, £176 flows into today's costs. Buying fuel and using fuel are different events.</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>The Fuel desk with the order instrument</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>Fuel order sum</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>briefing-fuel.html</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>aircraft_efficiency</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Week-2 shop, first comparison</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Two planes, one route</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>A Twin Otter and a Saab fly Dublin side by side; both gauges drain; a seat-row per plane.</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Which burned more per seat? Tap it.</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Litres per seat: the Saab 6.6, the Twin Otter 9.5 — bigger can be cheaper a seat, if it fills.</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>The comparison with the litres-per-seat widget</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>Second-plane decision</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>briefing-efficiency.html</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>event_weekend</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Announced event (day 22: the All Blacks)</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>One big Saturday</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>A normal Saturday: 62 Dublin dots. An event card slides onto the date; dots stream in to 124. Your two flights stay where they are.</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>What changed? Tap the day.</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Events change a market for a day; a weekend plan changes every Saturday.</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Can the planner respond to one date? → Upgrades question</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>day_override upgrade</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>briefing-event.html</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>seasons</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Chapter-1 review</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>A year of demand</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Twelve months; Geneva's bar grows in winter, Barcelona's in summer; Christmas and half-term markers.</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Drag a plane icon to the month you'd fly Geneva.</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Markets change through the year for different reasons; a weekly plan does not.</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>The Upgrades question (seasonal plans)</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>seasonal_plans upgrade</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>45</v>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>briefing-seasons.html</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>lease_money</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>6 Jan 2031, the 787 to lease</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Renting a plane</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>A 787; the price £12m against cash £1.5m; a rent meter ticks £6,000 a day.</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Slide the days: when does rent pass the price?</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Rent-or-buy: 12,000,000 ÷ 6,000 = 2,000 days. Rent keeps cash; buying keeps the plane.</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>The shop with Rent and (greyed) Buy</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Rent-or-buy sum</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>briefing-lease.html</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>profit_vs_cash</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Chapter 3, first overdrawn month or the 787 purchase</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Profit is not cash</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>The month's profit bar rises while the cash gauge falls: the money went into a plane and a full tank.</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Tap where the money went.</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Profit answers 'did we earn?'; cash answers 'can we pay?'. Both matter.</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>The Finance desk with the overdraft line</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Overdraft / buying outright</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>briefing-cash.html</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>D99: Show → Predict → Reveal → Use. Full screen, the interface darkened behind; the pupil advances by the interaction in beat 2, never by Next; a Pause &amp; discuss button at each stop for the teacher; a Replay from the Briefings shelf. Each is built as a separate HTML piece in the game's style (see the flight-time tutorial) and the game loads it at its trigger.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5040,7 +5689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5628,7 +6277,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7111,7 +7760,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7734,7 +8383,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
@@ -7747,7 +8395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8009,7 +8657,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10438,7 +11086,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11704,7 +12352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12747,7 +13395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13613,314 +14261,6 @@
       <c r="L20" s="13" t="inlineStr">
         <is>
           <t>live</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>landingFee</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>demandModifier</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>tendency</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>terminal</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>turnaroundMin</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>passengerCharge</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>LHR</t>
-        </is>
-      </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>London Heathrow</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="n">
-        <v>120</v>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>+15%</t>
-        </is>
-      </c>
-      <c r="E2" s="12" t="inlineStr">
-        <is>
-          <t>business</t>
-        </is>
-      </c>
-      <c r="F2" s="12" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="G2" s="12" t="n">
-        <v>35</v>
-      </c>
-      <c r="H2" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="I2" s="12" t="inlineStr">
-        <is>
-          <t>The only home airport at setup (D32)</t>
-        </is>
-      </c>
-      <c r="J2" s="12" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>LHR</t>
-        </is>
-      </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>London Heathrow</t>
-        </is>
-      </c>
-      <c r="C3" s="19" t="n">
-        <v>120</v>
-      </c>
-      <c r="D3" s="19" t="inlineStr">
-        <is>
-          <t>+15%</t>
-        </is>
-      </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>business</t>
-        </is>
-      </c>
-      <c r="F3" s="19" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="G3" s="19" t="n">
-        <v>55</v>
-      </c>
-      <c r="H3" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="I3" s="19" t="inlineStr">
-        <is>
-          <t>Removed 6 Oct (D32); row kept for its id</t>
-        </is>
-      </c>
-      <c r="J3" s="19" t="inlineStr">
-        <is>
-          <t>removed</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>LGW</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>London Gatwick</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="n">
-        <v>80</v>
-      </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>+5%</t>
-        </is>
-      </c>
-      <c r="E4" s="19" t="inlineStr">
-        <is>
-          <t>leisure</t>
-        </is>
-      </c>
-      <c r="F4" s="19" t="inlineStr">
-        <is>
-          <t>North</t>
-        </is>
-      </c>
-      <c r="G4" s="19" t="n">
-        <v>45</v>
-      </c>
-      <c r="H4" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="I4" s="19" t="inlineStr">
-        <is>
-          <t>Removed 6 Oct (D32); row kept for its id</t>
-        </is>
-      </c>
-      <c r="J4" s="19" t="inlineStr">
-        <is>
-          <t>removed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>LTN</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>London Luton</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="n">
-        <v>40</v>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>-5%</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr">
-        <is>
-          <t>leisure</t>
-        </is>
-      </c>
-      <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>Main</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="n">
-        <v>40</v>
-      </c>
-      <c r="H5" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="I5" s="15" t="inlineStr">
-        <is>
-          <t>Kept for the one-off April 2031 switch (fees_rise option 4). Needs a balance pass if taken.</t>
-        </is>
-      </c>
-      <c r="J5" s="15" t="inlineStr">
-        <is>
-          <t>later</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>MAN</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Manchester</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="n">
-        <v>60</v>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>mixed</t>
-        </is>
-      </c>
-      <c r="F6" s="19" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="G6" s="19" t="n">
-        <v>45</v>
-      </c>
-      <c r="H6" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="I6" s="19" t="inlineStr">
-        <is>
-          <t>Removed 6 Oct (D32); row kept for its id</t>
-        </is>
-      </c>
-      <c r="J6" s="19" t="inlineStr">
-        <is>
-          <t>removed</t>
         </is>
       </c>
     </row>
@@ -14368,6 +14708,314 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>landingFee</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>demandModifier</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>tendency</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>turnaroundMin</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>passengerCharge</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>London Heathrow</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>120</v>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>+15%</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="H2" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>The only home airport at setup (D32)</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>London Heathrow</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="n">
+        <v>120</v>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>+15%</t>
+        </is>
+      </c>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="n">
+        <v>55</v>
+      </c>
+      <c r="H3" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" s="19" t="inlineStr">
+        <is>
+          <t>Removed 6 Oct (D32); row kept for its id</t>
+        </is>
+      </c>
+      <c r="J3" s="19" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>London Gatwick</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>80</v>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>leisure</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="H4" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>Removed 6 Oct (D32); row kept for its id</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>LTN</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>London Luton</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>-5%</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>leisure</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="H5" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>Kept for the one-off April 2031 switch (fees_rise option 4). Needs a balance pass if taken.</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>later</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Manchester</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>Removed 6 Oct (D32); row kept for its id</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -15747,7 +16395,7 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>1.79</v>
+        <v>1.62</v>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
@@ -15761,16 +16409,16 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>Fuel £1.79 a litre.</t>
-        </is>
-      </c>
-      <c r="J23" s="13" t="inlineStr"/>
+          <t>Fuel £1.62 a litre.</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="n"/>
       <c r="K23" s="13" t="inlineStr">
         <is>
           <t>routes: mad; planes: e175, e190; mechanics: range check, services per day on a long leg, load factor as a percentage</t>
         </is>
       </c>
-      <c r="L23" s="13" t="inlineStr"/>
+      <c r="L23" s="13" t="n"/>
       <c r="M23" s="13" t="n"/>
       <c r="N23" s="13" t="inlineStr">
         <is>
@@ -15817,21 +16465,21 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>1.79</v>
+        <v>1.62</v>
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="H24" s="13" t="inlineStr"/>
-      <c r="I24" s="13" t="inlineStr"/>
-      <c r="J24" s="13" t="inlineStr"/>
-      <c r="K24" s="13" t="inlineStr"/>
-      <c r="L24" s="13" t="inlineStr"/>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="n"/>
+      <c r="J24" s="13" t="n"/>
+      <c r="K24" s="13" t="n"/>
+      <c r="L24" s="13" t="n"/>
       <c r="M24" s="13" t="n"/>
-      <c r="N24" s="13" t="inlineStr"/>
-      <c r="O24" s="13" t="inlineStr"/>
+      <c r="N24" s="13" t="n"/>
+      <c r="O24" s="13" t="n"/>
       <c r="P24" s="13" t="n"/>
       <c r="Q24" s="13" t="inlineStr">
         <is>
@@ -15867,7 +16515,7 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>1.79</v>
+        <v>1.62</v>
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
@@ -15879,17 +16527,17 @@
           <t>A jet burns in one trip what a Twin Otter burns in a week.</t>
         </is>
       </c>
-      <c r="I25" s="13" t="inlineStr"/>
-      <c r="J25" s="13" t="inlineStr"/>
-      <c r="K25" s="13" t="inlineStr"/>
-      <c r="L25" s="13" t="inlineStr"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
+      <c r="K25" s="13" t="n"/>
+      <c r="L25" s="13" t="n"/>
       <c r="M25" s="13" t="n"/>
       <c r="N25" s="13" t="inlineStr">
         <is>
           <t>fuel</t>
         </is>
       </c>
-      <c r="O25" s="13" t="inlineStr"/>
+      <c r="O25" s="13" t="n"/>
       <c r="P25" s="13" t="n"/>
       <c r="Q25" s="13" t="inlineStr">
         <is>
@@ -15925,7 +16573,7 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>1.79</v>
+        <v>1.62</v>
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
@@ -15937,13 +16585,13 @@
           <t>Red Kite announces Madrid flights from Luton.</t>
         </is>
       </c>
-      <c r="I26" s="13" t="inlineStr"/>
-      <c r="J26" s="13" t="inlineStr"/>
-      <c r="K26" s="13" t="inlineStr"/>
-      <c r="L26" s="13" t="inlineStr"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
+      <c r="K26" s="13" t="n"/>
+      <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="n"/>
-      <c r="N26" s="13" t="inlineStr"/>
-      <c r="O26" s="13" t="inlineStr"/>
+      <c r="N26" s="13" t="n"/>
+      <c r="O26" s="13" t="n"/>
       <c r="P26" s="13" t="n"/>
       <c r="Q26" s="13" t="inlineStr">
         <is>
@@ -15979,21 +16627,21 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>1.79</v>
+        <v>1.62</v>
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="H27" s="13" t="inlineStr"/>
-      <c r="I27" s="13" t="inlineStr"/>
-      <c r="J27" s="13" t="inlineStr"/>
-      <c r="K27" s="13" t="inlineStr"/>
-      <c r="L27" s="13" t="inlineStr"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="13" t="n"/>
+      <c r="L27" s="13" t="n"/>
       <c r="M27" s="13" t="n"/>
-      <c r="N27" s="13" t="inlineStr"/>
-      <c r="O27" s="13" t="inlineStr"/>
+      <c r="N27" s="13" t="n"/>
+      <c r="O27" s="13" t="n"/>
       <c r="P27" s="13" t="n"/>
       <c r="Q27" s="13" t="inlineStr">
         <is>
@@ -16029,25 +16677,25 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>1.79</v>
+        <v>1.62</v>
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="H28" s="13" t="inlineStr"/>
-      <c r="I28" s="13" t="inlineStr"/>
-      <c r="J28" s="13" t="inlineStr"/>
-      <c r="K28" s="13" t="inlineStr"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="13" t="n"/>
       <c r="L28" s="13" t="inlineStr">
         <is>
           <t>weekend multipliers (Settings)</t>
         </is>
       </c>
       <c r="M28" s="13" t="n"/>
-      <c r="N28" s="13" t="inlineStr"/>
-      <c r="O28" s="13" t="inlineStr"/>
+      <c r="N28" s="13" t="n"/>
+      <c r="O28" s="13" t="n"/>
       <c r="P28" s="13" t="n"/>
       <c r="Q28" s="13" t="inlineStr">
         <is>
@@ -16083,7 +16731,7 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>1.79</v>
+        <v>1.62</v>
       </c>
       <c r="G29" s="13" t="inlineStr">
         <is>
@@ -16095,8 +16743,8 @@
           <t>From next week the game runs a week at a time.</t>
         </is>
       </c>
-      <c r="I29" s="13" t="inlineStr"/>
-      <c r="J29" s="13" t="inlineStr"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
       <c r="K29" s="13" t="inlineStr">
         <is>
           <t>mechanics: weekly skips begin day 29</t>
@@ -17313,7 +17961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17588,22 +18236,23 @@
           <t>live</t>
         </is>
       </c>
-      <c r="L4" t="n">
-        <v>1.71</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1.87</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Analysts expect another small rise next week.</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
+      <c r="L4" s="13" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="M4" s="13" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>Tankers arriving early: prices expected to ease a little next week.</t>
+        </is>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="P4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="n">
@@ -17620,7 +18269,7 @@
         </is>
       </c>
       <c r="D5" s="12" t="n">
-        <v>1.79</v>
+        <v>1.62</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>1</v>
@@ -17639,28 +18288,29 @@
           <t>Clear</t>
         </is>
       </c>
-      <c r="J5" s="12" t="inlineStr"/>
+      <c r="J5" s="12" t="n"/>
       <c r="K5" s="12" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="L5" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="M5" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Steady rises continue.</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
+      <c r="L5" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="M5" s="13" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="N5" s="13" t="inlineStr">
+        <is>
+          <t>A quiet week; tankers arrived early. Prices expected to rise again as winter approaches.</t>
+        </is>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="P5" s="13" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="n">
@@ -17677,7 +18327,7 @@
         </is>
       </c>
       <c r="D6" s="12" t="n">
-        <v>1.86</v>
+        <v>1.74</v>
       </c>
       <c r="E6" s="12" t="n">
         <v>1</v>
@@ -17696,28 +18346,29 @@
           <t>Storm over the Irish Sea</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr"/>
+      <c r="J6" s="12" t="n"/>
       <c r="K6" s="12" t="inlineStr">
         <is>
           <t>live</t>
         </is>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="13" t="n">
         <v>1.89</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="13" t="n">
         <v>2.05</v>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N6" s="13" t="inlineStr">
         <is>
           <t>Little change expected.</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="13" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
+      <c r="P6" s="13" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="n">
@@ -36813,7 +37464,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -38850,7 +39501,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -39311,7 +39962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -39729,7 +40380,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -39958,7 +40609,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40311,7 +40962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -42830,7 +43481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D162"/>
+  <dimension ref="A1:D180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -44797,12 +45448,12 @@
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>selected route, else all routes</t>
+          <t>follows the selected flight's route; otherwise route tabs (each route · All)</t>
         </is>
       </c>
       <c r="C95" s="13" t="inlineStr">
         <is>
-          <t>D66: the demand-through-the-day strip shows the selected or hovered route's own five bands (Archetypes shares); with nothing selected, the sum across open routes.</t>
+          <t>D100: the strip header always names what it shows ('Madrid · people who want to fly at £170'); 'All' is a tab, never the silent default.</t>
         </is>
       </c>
       <c r="D95" s="13" t="inlineStr">
@@ -46200,6 +46851,398 @@
         </is>
       </c>
       <c r="D162" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="13" t="inlineStr">
+        <is>
+          <t>adaptToOnlyFlight</t>
+        </is>
+      </c>
+      <c r="B163" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C163" s="13" t="inlineStr">
+        <is>
+          <t>D101: when time-locked passengers want a band with no service on their route, this share of them take the nearest service on that route instead. Fixes one-flight routes that could never fill (Marrakech: 76 → about 87 wanting the 06:00); timing still matters wherever a route has more than one service.</t>
+        </is>
+      </c>
+      <c r="D163" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="13" t="inlineStr">
+        <is>
+          <t>demandShapeDisplay</t>
+        </is>
+      </c>
+      <c r="B164" s="13" t="inlineStr">
+        <is>
+          <t>route demand by band, flexible shown separately; the selected flight's catchable slice highlighted</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="inlineStr">
+        <is>
+          <t>D101: the route card and the strip show demand as a shape across the day plus the 'any time' passengers, and when a flight is selected the part it can catch lights up (its band's locked passengers + the flexible ones not taken by earlier flights + the adapters).</t>
+        </is>
+      </c>
+      <c r="D164" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="13" t="inlineStr">
+        <is>
+          <t>flightTimeDecay</t>
+        </is>
+      </c>
+      <c r="B165" s="13" t="inlineStr">
+        <is>
+          <t>per kind of sum, whole game: Calculate twice, then Build, then Model</t>
+        </is>
+      </c>
+      <c r="C165" s="13" t="inlineStr">
+        <is>
+          <t>D101: flight-time sums count once for the whole game, not per aircraft and route; a plane already flying a route is never asked about it.</t>
+        </is>
+      </c>
+      <c r="D165" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="13" t="inlineStr">
+        <is>
+          <t>timeAnswerFormat</t>
+        </is>
+      </c>
+      <c r="B166" s="13" t="inlineStr">
+        <is>
+          <t>hours + minutes (selector 0, 15, 30, 45)</t>
+        </is>
+      </c>
+      <c r="C166" s="13" t="inlineStr">
+        <is>
+          <t>D101: no decimal hours in answers or questions; '225 km ÷ 900 km/h = ? h ? min'.</t>
+        </is>
+      </c>
+      <c r="D166" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="13" t="inlineStr">
+        <is>
+          <t>flightTimesTable</t>
+        </is>
+      </c>
+      <c r="B167" s="13" t="inlineStr">
+        <is>
+          <t>fixed-width columns; the active sum in the instrument below with its cell highlighted; a 'time saved' column between aircraft</t>
+        </is>
+      </c>
+      <c r="C167" s="13" t="inlineStr">
+        <is>
+          <t>D101: e.g. 'Twin Otter 1 h 30 → Saab 1 h: 30 min faster'.</t>
+        </is>
+      </c>
+      <c r="D167" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="13" t="inlineStr">
+        <is>
+          <t>weekPlanTutorial</t>
+        </is>
+      </c>
+      <c r="B168" s="13" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="C168" s="13" t="inlineStr">
+        <is>
+          <t>D101: the week-5 'Planning a whole week' tutorial goes; a one-line notice says the game now runs a week at a time.</t>
+        </is>
+      </c>
+      <c r="D168" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="13" t="inlineStr">
+        <is>
+          <t>redMeans</t>
+        </is>
+      </c>
+      <c r="B169" s="13" t="inlineStr">
+        <is>
+          <t>only genuinely bad or urgent: an invalid timetable, a plane that can't reach a route, a real loss, a disruption</t>
+        </is>
+      </c>
+      <c r="C169" s="13" t="inlineStr">
+        <is>
+          <t>D101 amends D95: unserved demand and forecast variance are information, never red.</t>
+        </is>
+      </c>
+      <c r="D169" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="13" t="inlineStr">
+        <is>
+          <t>opportunityDisplay</t>
+        </is>
+      </c>
+      <c r="B170" s="13" t="inlineStr">
+        <is>
+          <t>quiet type with an 'opportunity' label; gold only on the single biggest opportunity on a screen</t>
+        </is>
+      </c>
+      <c r="C170" s="13" t="inlineStr">
+        <is>
+          <t>D101: keeps gold rare (D95).</t>
+        </is>
+      </c>
+      <c r="D170" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="13" t="inlineStr">
+        <is>
+          <t>resultsFraming</t>
+        </is>
+      </c>
+      <c r="B171" s="13" t="inlineStr">
+        <is>
+          <t>lead with the result and the comparison with last week; variance with its reasons; 'passengers we couldn't carry' totalled once; cash change as profit − fuel bought</t>
+        </is>
+      </c>
+      <c r="C171" s="13" t="inlineStr">
+        <is>
+          <t>D101.</t>
+        </is>
+      </c>
+      <c r="D171" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="13" t="inlineStr">
+        <is>
+          <t>flightInspector</t>
+        </is>
+      </c>
+      <c r="B172" s="13" t="inlineStr">
+        <is>
+          <t>fixed bar under the timetable</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="inlineStr">
+        <is>
+          <t>D101: Earlier · Later · Route · Fare · Days · Aircraft · Remove; never moves; the focus rail marks the selected block.</t>
+        </is>
+      </c>
+      <c r="D172" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="13" t="inlineStr">
+        <is>
+          <t>activeRoutesCollapsible</t>
+        </is>
+      </c>
+      <c r="B173" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C173" s="13" t="inlineStr">
+        <is>
+          <t>D101: collapses to one line ('7 routes · 9 flights a day · 98% filled · 2 need attention') with route chips; opens with a tap.</t>
+        </is>
+      </c>
+      <c r="D173" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="13" t="inlineStr">
+        <is>
+          <t>weekGraphDefault</t>
+        </is>
+      </c>
+      <c r="B174" s="13" t="inlineStr">
+        <is>
+          <t>weekly history (profit per week so far, projection as a faint marker); 'this week by day' as a tab</t>
+        </is>
+      </c>
+      <c r="C174" s="13" t="inlineStr">
+        <is>
+          <t>D101.</t>
+        </is>
+      </c>
+      <c r="D174" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="13" t="inlineStr">
+        <is>
+          <t>dailyColourLimit</t>
+        </is>
+      </c>
+      <c r="B175" s="13" t="inlineStr">
+        <is>
+          <t>at most two a week; never the same item twice in a row; no duplicate lines</t>
+        </is>
+      </c>
+      <c r="C175" s="13" t="inlineStr">
+        <is>
+          <t>D101: tightens the DailyColour rule after a week showed four and a repeat.</t>
+        </is>
+      </c>
+      <c r="D175" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="13" t="inlineStr">
+        <is>
+          <t>comingUp</t>
+        </is>
+      </c>
+      <c r="B176" s="13" t="inlineStr">
+        <is>
+          <t>Roadmap sheet</t>
+        </is>
+      </c>
+      <c r="C176" s="13" t="inlineStr">
+        <is>
+          <t>D101: a 'Coming up' strip on Home (NOW · NEXT · LATER) and one line at the end of each review about next week. Planner upgrades are never named in advance.</t>
+        </is>
+      </c>
+      <c r="D176" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="13" t="inlineStr">
+        <is>
+          <t>aircraftWorthCheck</t>
+        </is>
+      </c>
+      <c r="B177" s="13" t="inlineStr">
+        <is>
+          <t>inside the comparison, not a separate page</t>
+        </is>
+      </c>
+      <c r="C177" s="13" t="inlineStr">
+        <is>
+          <t>D101: choosing a plane on 'Which aircraft should we add?' opens its worth check in place: WHY (the routes leaving people behind, with numbers) · WORK IT OUT (one full flight at the route's current fare) · WHAT IT MEANS (full-flight money → extra profit a day → payback, revealed one by one after the answer, payback as a coin bar). No numbered steps, no 'recommended routes', no sum counter; Give me a hint.</t>
+        </is>
+      </c>
+      <c r="D177" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="13" t="inlineStr">
+        <is>
+          <t>teacherTestMode</t>
+        </is>
+      </c>
+      <c r="B178" s="13" t="inlineStr">
+        <is>
+          <t>teacher panel, behind the PIN; amber TEST MODE bar; Answer · Answer all · Auto-plan · Run week/month · Skip briefing · Jump to… · Show the answer · Event now</t>
+        </is>
+      </c>
+      <c r="C178" s="13" t="inlineStr">
+        <is>
+          <t>D102: for testing screens without playing every sum. Nothing in test mode reaches the record, milestones or sum numbering; test airlines saved separately and labelled TEST. Jump-to points along the Steady path: Launch Day, weeks 2, 3, 4, 5, 7, 9, December, January 2031, June 2031, chapter 3, chapter 4. Shortcuts Ctrl+Shift+T (tools), Ctrl+Shift+A (answer), Ctrl+Shift+R (run).</t>
+        </is>
+      </c>
+      <c r="D178" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="13" t="inlineStr">
+        <is>
+          <t>waitCostLine</t>
+        </is>
+      </c>
+      <c r="B179" s="13" t="inlineStr">
+        <is>
+          <t>idle days × day cost</t>
+        </is>
+      </c>
+      <c r="C179" s="13" t="inlineStr">
+        <is>
+          <t>D100: on Buy now or wait, per plane: 'Its best work starts {date} ({route}). Bought today, it costs £{dayCost} a day for {days} days first: £{total}', against its earnings meanwhile. A Build the first time.</t>
+        </is>
+      </c>
+      <c r="D179" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="13" t="inlineStr">
+        <is>
+          <t>aircraftCardMeasure</t>
+        </is>
+      </c>
+      <c r="B180" s="13" t="inlineStr">
+        <is>
+          <t>extra profit for the airline (incremental), one measure on the whole screen</t>
+        </is>
+      </c>
+      <c r="C180" s="13" t="inlineStr">
+        <is>
+          <t>D100: the cards, the waterfall, 'What the extra money buys' and 'Where could it fly?' all use the airline's extra profit against today's plan; the waterfall must add up line by line (show snacks if included); the route's current fare unless a card says otherwise; 'What you give up' written per plane from its own figures.</t>
+        </is>
+      </c>
+      <c r="D180" s="13" t="inlineStr">
         <is>
           <t>live</t>
         </is>
@@ -46817,7 +47860,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
@@ -47393,7 +48435,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
@@ -47407,6 +48448,342 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>when</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>now / next / later line</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>shown from</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Week 3</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>New routes: Amsterdam, Frankfurt, Geneva, Barcelona</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>day 8</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Week 4</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Medium haul: Madrid, and your first jets</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>day 15</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Marrakech — and the game runs a week at a time</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>day 22</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Brussels, Berlin and Milan</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>day 29</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Week 7</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Rome and Lisbon</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>day 36</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Week 9</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Bigger jets in the shop: the A220, A320 and 737</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>day 50</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Week 9</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Athens and Istanbul</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>day 50</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>A month at a time — and the chapter review</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>day 78</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>January 2031</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Long haul: New York, Dubai, and the 787</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>day 85</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>January 2031</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Your star rating goes public; what sort of airline are you?</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>day 106</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>June 2031</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Delhi: the first flight too far for one day</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>day 240</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>September 2031</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Buying big planes outright; Tokyo and Cape Town</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>day 330</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>September 2032</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>The ultimate plane</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>day 700</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>D101: Home shows the current stage (NOW), the next item (NEXT) and one or two after it (LATER), each with a greyed silhouette until it arrives. Planner upgrades (Upgrades sheet) are never listed: the pupil discovers the need.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47739,653 +49116,10 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>D98: the review shows dataShown, then asks the question with the three options as cards (the right one first in the sheet, shuffled on screen); from freeTextFrom the pupil writes the requirement in a sentence and picks the card it matches. Granting: a result plate 'Operations request · Planner upgrade approved: …'. Fallback: the systems team proposes it with the same card. The data never waits: the feature exists in the engine from day one and is simply switched on for the pupil.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>briefingId</t>
-        </is>
-      </c>
-      <c r="B1" s="20" t="inlineStr">
-        <is>
-          <t>trigger</t>
-        </is>
-      </c>
-      <c r="C1" s="20" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="D1" s="20" t="inlineStr">
-        <is>
-          <t>beat1 (show)</t>
-        </is>
-      </c>
-      <c r="E1" s="20" t="inlineStr">
-        <is>
-          <t>beat2 (predict: the pupil does…)</t>
-        </is>
-      </c>
-      <c r="F1" s="20" t="inlineStr">
-        <is>
-          <t>beat3 (reveal)</t>
-        </is>
-      </c>
-      <c r="G1" s="20" t="inlineStr">
-        <is>
-          <t>beat4 (use)</t>
-        </is>
-      </c>
-      <c r="H1" s="20" t="inlineStr">
-        <is>
-          <t>leadsInto</t>
-        </is>
-      </c>
-      <c r="I1" s="20" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
-      <c r="J1" s="20" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="K1" s="20" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>fare_lever</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>Launch Day, the fare chips</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>What a fare does</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Nineteen passenger dots and a £ meter. The fare slides from £80 to £90 to £100; the meter per passenger rises as dots fade.</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>Drag the fare yourself; predict: more or fewer dots at £100?</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>Revenue = passengers × fare: both move. At £100 Paris wants 44, not 50 — two planes still fill.</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>Back to the chips with the three revenue figures</t>
-        </is>
-      </c>
-      <c r="H2" s="13" t="inlineStr">
-        <is>
-          <t>Launch Day sum 1</t>
-        </is>
-      </c>
-      <c r="I2" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="J2" s="13" t="inlineStr">
-        <is>
-          <t>briefing-fare.html</t>
-        </is>
-      </c>
-      <c r="K2" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>rival_split</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Thu, week 1 (Red Kite)</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>Customers have a choice</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>62 Dublin dots; a red-kite plane lands beside yours; its price tag reads £50.</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>Slide your fare; watch dots cross to Red Kite: 1 in 10 per £10.</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>The switching rule in one line; advertising halves it.</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>The Red Kite decision with the sum on it</t>
-        </is>
-      </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>Red Kite card</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>briefing-rival.html</t>
-        </is>
-      </c>
-      <c r="K3" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>full_route</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Week-1 review</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>More demand than seats</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Passenger dots arrive at the terminal; 57 board three Twin Otters; the rest stay on the apron.</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>Click the dots left behind; how many?</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>High demand is not profit if you cannot carry people: a bigger plane, another plane, or a higher fare.</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>The capacity observation and Compare aircraft</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>Week-2 decision</t>
-        </is>
-      </c>
-      <c r="I4" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
-        <is>
-          <t>briefing-capacity.html</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>weekend_demand</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Week-2 review</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>Weekdays and weekends</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Mon–Sun bars grow for Dublin; business icons fill weekdays, families the weekend.</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>Click the days that look different.</t>
-        </is>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>Why: business travel builds on weekdays; leisure swells at the weekend. Your timetable appears underneath — the same every day.</t>
-        </is>
-      </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>Does the planner fit what the passengers do? → the Upgrades question</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>weekend_schedules upgrade</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="n">
-        <v>45</v>
-      </c>
-      <c r="J5" s="13" t="inlineStr">
-        <is>
-          <t>briefing-weekend.html</t>
-        </is>
-      </c>
-      <c r="K5" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>fuel_cash_tank_profit</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>First Fuel desk visit (day 8)</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>Cash, tank, profit</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Three gauges: cash £12,409, tank 0 L, profit today. Press Buy 7,000 L: cash flows into the tank; profit does not move.</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>Press Buy yourself; then: what changed? (tap the gauge)</t>
-        </is>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>A Twin Otter departs for Paris: 120 L drains, £176 flows into today's costs. Buying fuel and using fuel are different events.</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>The Fuel desk with the order instrument</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>Fuel order sum</t>
-        </is>
-      </c>
-      <c r="I6" s="13" t="n">
-        <v>50</v>
-      </c>
-      <c r="J6" s="13" t="inlineStr">
-        <is>
-          <t>briefing-fuel.html</t>
-        </is>
-      </c>
-      <c r="K6" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>aircraft_efficiency</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Week-2 shop, first comparison</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>Two planes, one route</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>A Twin Otter and a Saab fly Dublin side by side; both gauges drain; a seat-row per plane.</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>Which burned more per seat? Tap it.</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>Litres per seat: the Saab 6.6, the Twin Otter 9.5 — bigger can be cheaper a seat, if it fills.</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>The comparison with the litres-per-seat widget</t>
-        </is>
-      </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>Second-plane decision</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>briefing-efficiency.html</t>
-        </is>
-      </c>
-      <c r="K7" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>event_weekend</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Announced event (day 22: the All Blacks)</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>One big Saturday</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>A normal Saturday: 62 Dublin dots. An event card slides onto the date; dots stream in to 124. Your two flights stay where they are.</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>What changed? Tap the day.</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>Events change a market for a day; a weekend plan changes every Saturday.</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Can the planner respond to one date? → Upgrades question</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>day_override upgrade</t>
-        </is>
-      </c>
-      <c r="I8" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>briefing-event.html</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>seasons</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Chapter-1 review</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>A year of demand</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Twelve months; Geneva's bar grows in winter, Barcelona's in summer; Christmas and half-term markers.</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>Drag a plane icon to the month you'd fly Geneva.</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>Markets change through the year for different reasons; a weekly plan does not.</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>The Upgrades question (seasonal plans)</t>
-        </is>
-      </c>
-      <c r="H9" s="13" t="inlineStr">
-        <is>
-          <t>seasonal_plans upgrade</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="n">
-        <v>45</v>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>briefing-seasons.html</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>lease_money</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>6 Jan 2031, the 787 to lease</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>Renting a plane</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>A 787; the price £12m against cash £1.5m; a rent meter ticks £6,000 a day.</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>Slide the days: when does rent pass the price?</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>Rent-or-buy: 12,000,000 ÷ 6,000 = 2,000 days. Rent keeps cash; buying keeps the plane.</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>The shop with Rent and (greyed) Buy</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>Rent-or-buy sum</t>
-        </is>
-      </c>
-      <c r="I10" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="J10" s="13" t="inlineStr">
-        <is>
-          <t>briefing-lease.html</t>
-        </is>
-      </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>profit_vs_cash</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Chapter 3, first overdrawn month or the 787 purchase</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>Profit is not cash</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>The month's profit bar rises while the cash gauge falls: the money went into a plane and a full tank.</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>Tap where the money went.</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>Profit answers 'did we earn?'; cash answers 'can we pay?'. Both matter.</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>The Finance desk with the overdraft line</t>
-        </is>
-      </c>
-      <c r="H11" s="13" t="inlineStr">
-        <is>
-          <t>Overdraft / buying outright</t>
-        </is>
-      </c>
-      <c r="I11" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>briefing-cash.html</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>D99: Show → Predict → Reveal → Use. Full screen, the interface darkened behind; the pupil advances by the interaction in beat 2, never by Next; a Pause &amp; discuss button at each stop for the teacher; a Replay from the Briefings shelf. Each is built as a separate HTML piece in the game's style (see the flight-time tutorial) and the game loads it at its trigger.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Briefings review PDF; fare slider easier to move; Snacks on board dropped
- docs/Briefings-Review.pdf: Bertie's notes on every briefing, what each
  note asks for, the words on screen and the screenshots (fare briefing
  included), for ChatGPT and Claude Design
- What a fare does: the slider has a bigger touch area and each fare
  under it can be pressed
- Workbook: cabin_sales briefing marked dropped; re-imported and rebuilt
- fare_lever screenshots added to docs/screenshots/briefings-review

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013x87PezhtynWHJHngTWCer
</commit_message>
<xml_diff>
--- a/data/Airline-World-Workbook.xlsx
+++ b/data/Airline-World-Workbook.xlsx
@@ -2234,6 +2234,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
@@ -2359,7 +2360,7 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Launch Day, before the cabin-sales Builds</t>
+          <t>Launch Day, before the cabin-sales Builds · Bertie, 20 Oct 2026: not needed (dropped)</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -2402,7 +2403,7 @@
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4682,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
         <is>
@@ -10372,7 +10372,6 @@
         </is>
       </c>
     </row>
-    <row r="103"/>
     <row r="104">
       <c r="A104" s="17" t="inlineStr">
         <is>
@@ -12215,7 +12214,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
@@ -51628,7 +51626,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
         <is>

</xml_diff>